<commit_message>
docs: agregar 4 perfiles nuevos a prospección LinkedIn
</commit_message>
<xml_diff>
--- a/docs/tracker-prospectos-neggo.xlsx
+++ b/docs/tracker-prospectos-neggo.xlsx
@@ -1783,7 +1783,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K10"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="7" min="1" max="1"/>
@@ -2196,6 +2196,226 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="16" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>Adriana Giraldo Mejia</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>Comercio directo</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>CEO, AGL Eventos Empresariales (también Directora Ejecutiva, Asociación Antioqueña de Otorrinolaringología)</t>
+        </is>
+      </c>
+      <c r="E11" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/adriana-giraldo-mejia-003259159/</t>
+        </is>
+      </c>
+      <c r="F11" s="16" t="inlineStr">
+        <is>
+          <t>Juan Sebastián y Lucía</t>
+        </is>
+      </c>
+      <c r="G11" s="16" t="inlineStr">
+        <is>
+          <t>Categoría ICP #5 (eventos) — CEO de empresa de eventos empresariales en Medellín</t>
+        </is>
+      </c>
+      <c r="H11" s="16" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I11" s="16" t="inlineStr">
+        <is>
+          <t>Mensaje armado</t>
+        </is>
+      </c>
+      <c r="J11" s="16" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="K11" s="16" t="inlineStr">
+        <is>
+          <t>Perfil marcado "en busca de empleo" pero rol vigente es CEO de AGL Eventos — verificar interés real antes de insistir</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="16" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>Angela María Vélez Toro</t>
+        </is>
+      </c>
+      <c r="C12" s="16" t="inlineStr">
+        <is>
+          <t>Comercio directo</t>
+        </is>
+      </c>
+      <c r="D12" s="16" t="inlineStr">
+        <is>
+          <t>Directora clínica, Clínica Odontoser</t>
+        </is>
+      </c>
+      <c r="E12" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/angela-mar%C3%ADa-v%C3%A9lez-toro-b738681ba/</t>
+        </is>
+      </c>
+      <c r="F12" s="16" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="G12" s="16" t="inlineStr">
+        <is>
+          <t>Categoría ICP #1 (odontología) — Directora de clínica dental en Medellín</t>
+        </is>
+      </c>
+      <c r="H12" s="16" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I12" s="16" t="inlineStr">
+        <is>
+          <t>Mensaje armado</t>
+        </is>
+      </c>
+      <c r="J12" s="16" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="K12" s="16" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="16" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>Michael Andrés García Pérez</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>Conector</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>Consultor Empresarial / Director Comercial — 20 años en estrategia comercial y crecimiento de pymes</t>
+        </is>
+      </c>
+      <c r="E13" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/michael-andr%C3%A9s-garc%C3%ADa-p%C3%A9rez-1aa56252/</t>
+        </is>
+      </c>
+      <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>Daniel Betancur</t>
+        </is>
+      </c>
+      <c r="G13" s="16" t="inlineStr">
+        <is>
+          <t>Consultor independiente enfocado en pymes — candidato natural para referir negocios</t>
+        </is>
+      </c>
+      <c r="H13" s="16" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I13" s="16" t="inlineStr">
+        <is>
+          <t>Mensaje armado</t>
+        </is>
+      </c>
+      <c r="J13" s="16" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="K13" s="16" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>Carolina Zuleta</t>
+        </is>
+      </c>
+      <c r="C14" s="16" t="inlineStr">
+        <is>
+          <t>Constructora</t>
+        </is>
+      </c>
+      <c r="D14" s="16" t="inlineStr">
+        <is>
+          <t>Gerente Comercial / Estructuración y Gerencia de Proyectos, Convel S.A.S (sector inmobiliario y construcción)</t>
+        </is>
+      </c>
+      <c r="E14" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/carolina-zuleta/</t>
+        </is>
+      </c>
+      <c r="F14" s="16" t="inlineStr">
+        <is>
+          <t>Andrés Escobar Uribe</t>
+        </is>
+      </c>
+      <c r="G14" s="16" t="inlineStr">
+        <is>
+          <t>Constructora real, rol de estructuración de negocios — mensaje informal, sin pitch (fase 2 aún no arranca)</t>
+        </is>
+      </c>
+      <c r="H14" s="16" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I14" s="16" t="inlineStr">
+        <is>
+          <t>Mensaje armado</t>
+        </is>
+      </c>
+      <c r="J14" s="16" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="K14" s="16" t="inlineStr">
+        <is>
+          <t>Solo conversación exploratoria — no formal, regla de estrategia-adquisicion sección 9</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:K2"/>

</xml_diff>

<commit_message>
docs: agregar 3 perfiles nuevos a prospección LinkedIn
</commit_message>
<xml_diff>
--- a/docs/tracker-prospectos-neggo.xlsx
+++ b/docs/tracker-prospectos-neggo.xlsx
@@ -1783,7 +1783,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K14"/>
+  <dimension ref="A1:K17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="7" min="1" max="1"/>
@@ -2359,7 +2359,7 @@
       </c>
       <c r="K13" s="16" t="n"/>
     </row>
-    <row r="14">
+    <row r="14" s="7">
       <c r="A14" s="16" t="inlineStr">
         <is>
           <t>2026-07-31</t>
@@ -2413,6 +2413,169 @@
       <c r="K14" s="16" t="inlineStr">
         <is>
           <t>Solo conversación exploratoria — no formal, regla de estrategia-adquisicion sección 9</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" s="7">
+      <c r="A15" s="16" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>María Azaín Ayala</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>Comercio directo</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>Cirujana plástica, estética y reconstructiva (práctica propia)</t>
+        </is>
+      </c>
+      <c r="E15" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/doctora-maria-azain/</t>
+        </is>
+      </c>
+      <c r="F15" s="16" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="G15" s="16" t="inlineStr">
+        <is>
+          <t>Categoría ICP #1 (cirugía estética) — práctica propia en Medellín</t>
+        </is>
+      </c>
+      <c r="H15" s="16" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I15" s="16" t="inlineStr">
+        <is>
+          <t>Mensaje armado</t>
+        </is>
+      </c>
+      <c r="J15" s="16" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="K15" s="16" t="n"/>
+    </row>
+    <row r="16" s="7">
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B16" s="16" t="inlineStr">
+        <is>
+          <t>Esteban Cadavid</t>
+        </is>
+      </c>
+      <c r="C16" s="16" t="inlineStr">
+        <is>
+          <t>Conector</t>
+        </is>
+      </c>
+      <c r="D16" s="16" t="inlineStr">
+        <is>
+          <t>Consultor Financiero para PYMES — contenido "Hablemos de tu negocio" (2.991 seguidores)</t>
+        </is>
+      </c>
+      <c r="E16" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/estebancadavid/</t>
+        </is>
+      </c>
+      <c r="F16" s="16" t="inlineStr">
+        <is>
+          <t>Yady Alexandra Anzueta Duarte y Carlos Guayara</t>
+        </is>
+      </c>
+      <c r="G16" s="16" t="inlineStr">
+        <is>
+          <t>Consultor financiero independiente para pymes en Medellín — candidato natural para referir negocios</t>
+        </is>
+      </c>
+      <c r="H16" s="16" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I16" s="16" t="inlineStr">
+        <is>
+          <t>Mensaje armado</t>
+        </is>
+      </c>
+      <c r="J16" s="16" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="K16" s="16" t="n"/>
+    </row>
+    <row r="17" s="7">
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>Sandra Milena Holguin Ramirez</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>Banco</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>Gerente Transaccional Senior, BBVA Regional Antioquia-Medellín</t>
+        </is>
+      </c>
+      <c r="E17" s="16" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/sandra-milena-holguin-ramirez-12a2a61ba/</t>
+        </is>
+      </c>
+      <c r="F17" s="16" t="inlineStr">
+        <is>
+          <t>Yady Alexandra Anzueta Duarte y Harry Viasús</t>
+        </is>
+      </c>
+      <c r="G17" s="16" t="inlineStr">
+        <is>
+          <t>Banco real, cash management + estructuración de negocios — mensaje informal, sin pitch (fase 3 bloqueada)</t>
+        </is>
+      </c>
+      <c r="H17" s="16" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="I17" s="16" t="inlineStr">
+        <is>
+          <t>Mensaje armado</t>
+        </is>
+      </c>
+      <c r="J17" s="16" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="K17" s="16" t="inlineStr">
+        <is>
+          <t>Solo conversación exploratoria — no formal, regla de estrategia-adquisicion sección 10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: agregar columnas Perfil LinkedIn/Contactos en común/Próxima acción al tracker
</commit_message>
<xml_diff>
--- a/docs/tracker-prospectos-neggo.xlsx
+++ b/docs/tracker-prospectos-neggo.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -38,6 +38,10 @@
     <font>
       <name val="Arial"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -65,7 +69,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -73,6 +77,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1429,7 +1434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:K13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1463,22 +1468,37 @@
           <t>Cargo/Empresa</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Perfil LinkedIn</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Contactos en común</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Gancho real</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Mensaje armado</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>Próxima acción</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Estado (Armado/Enviado por Jhey)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Notas</t>
         </is>
@@ -1505,22 +1525,33 @@
           <t>Fundador — BTODigital (marketing digital y soluciones tecnológicas), Medellín</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>No capturado (corrida previa a la corrección del 3 ago)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Fundador de agencia con clientes pyme en Medellín — perfil público de LinkedIn</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Hola, Carlos. Sigo tu trabajo al frente de BTODigital con pymes de Medellín. Estoy construyendo Neggo, una plataforma que conecta negocios de la ciudad con clientes verificados que ya están buscando su servicio, con pago por resultado (CPL). Creo que complementa —no compite con— el marketing que haces para tus clientes: tú construyes la marca, nosotros entregamos demanda ya calificada. ¿Te interesa conversarlo 10 minutos?</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>Armado</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>Mensaje listo — pendiente de envío por Jhey (no enviado)</t>
         </is>
@@ -1547,22 +1578,33 @@
           <t>Consultor y mentor de emprendedores — Taglic Digital, Medellín</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>No capturado (corrida previa a la corrección del 3 ago)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Consultor de marketing digital y mentor de emprendedores en Medellín — perfil público de LinkedIn</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Hola, Juan. Vi tu trabajo como consultor y mentor de emprendedores desde Taglic Digital en Medellín. Estoy construyendo Neggo, una plataforma que conecta negocios locales con clientes verificados que piden contacto directo, pagando solo por resultado. Muchos de los emprendedores que acompañas podrían ser justo el perfil. ¿Te cuento en 10 minutos y me das tu mirada?</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>Armado</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>Mensaje listo — pendiente de envío por Jhey (no enviado)</t>
         </is>
@@ -1589,22 +1631,33 @@
           <t>Implementador de CRM y sistemas de ventas (integración WhatsApp)</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>No capturado (corrida previa a la corrección del 3 ago)</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>Implementa CRM y sistemas de ventas con WhatsApp para equipos comerciales — perfil público de LinkedIn. OJO: ciudad no confirmada</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Hola, Ramón. Vi que implementas CRM y sistemas de ventas con integración de WhatsApp. Estoy construyendo Neggo, un marketplace en Medellín que entrega leads verificados a negocios locales — los equipos que tú montas en CRM son exactamente quienes reciben esos leads. Veo una conexión natural entre lo tuyo y lo nuestro. ¿Lo conversamos 10 minutos?</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>Armado</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>VERIFICAR ciudad en el perfil antes de enviar — no confirmada en la búsqueda. Mensaje listo — pendiente de envío por Jhey (no enviado)</t>
         </is>
@@ -1631,22 +1684,33 @@
           <t>Gerente Comercial y Desarrollo de Negocios — Elige Realty Group, Medellín</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>No capturado (corrida previa a la corrección del 3 ago)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>5+ años en gestión comercial inmobiliaria en Medellín — perfil público de LinkedIn</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>Hola, Manuela. Vi tu rol comercial en Elige Realty Group en Medellín. Estoy construyendo Neggo, una plataforma que conecta compradores verificados (con score financiero) con constructoras y comercios de la ciudad. Aún estamos en etapa temprana, y me encantaría conocer tu mirada sobre cómo llegan hoy los leads a los proyectos inmobiliarios en Medellín — sin ningún compromiso comercial, solo aprender de quien está en el terreno. ¿Te sumo a un café virtual de 15 minutos?</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>Armado</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>EXPLORATORIO — sin pitch formal ni CTA de registro (regla secciones 9-10). Mensaje listo — pendiente de envío por Jhey (no enviado)</t>
         </is>
@@ -1673,22 +1737,33 @@
           <t>Gerente de Proyectos — Promotora &amp; Constructora de Proyectos SAS, Medellín</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>No capturado (corrida previa a la corrección del 3 ago)</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Rol reciente de Gerente de Proyectos en promotora/constructora de Medellín — perfil público de LinkedIn</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>Hola, Juan. Vi tu paso a Gerente de Proyectos en Promotora &amp; Constructora de Proyectos. Estoy construyendo Neggo, una plataforma de Medellín que conecta compradores verificados con constructoras por ciudad, estrato y presupuesto. Estamos en etapa temprana y me interesa entender cómo captan compradores hoy los proyectos en la ciudad — conversación sin compromiso, de fundador a alguien que vive el negocio. ¿Tienes 15 minutos esta semana?</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>Armado</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>EXPLORATORIO — sin pitch formal. Mensaje listo — pendiente de envío por Jhey (no enviado)</t>
         </is>
@@ -1715,22 +1790,33 @@
           <t>Gerente de sucursal — Bancolombia, Medellín (experiencia en banca empresarial y pymes)</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>No capturado (corrida previa a la corrección del 3 ago)</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Gerente de sucursal Bancolombia en Medellín con experiencia en banca pyme — perfil público de LinkedIn</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>Hola, Mauricio. Vi tu experiencia liderando sucursal y banca pyme en Bancolombia en Medellín. Estoy construyendo Neggo, una plataforma de la ciudad que conecta clientes verificados con negocios y entidades financieras. Estamos en etapa temprana y me encantaría conocer tu perspectiva sobre cómo la banca ve hoy la adquisición digital de clientes — conversación informal, sin ninguna propuesta de por medio. ¿Te invito un café (virtual o presencial) de 15 minutos?</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>Armado</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>EXPLORATORIO — regla dura: cero pitch formal a bancos hasta cerrar los 3 pendientes de seguridad. Mensaje listo — pendiente de envío por Jhey (no enviado)</t>
         </is>
@@ -1757,22 +1843,33 @@
           <t>Gerente Banca Empresarial — Banco de Occidente, Medellín</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>No capturado (corrida previa a la corrección del 3 ago)</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Gerente de Banca Empresarial en Banco de Occidente, Medellín — perfil público de LinkedIn</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>Hola, María de los Ángeles. Vi tu rol en Banca Empresarial de Banco de Occidente en Medellín. Estoy construyendo Neggo, una plataforma local que conecta clientes finales verificados con negocios y entidades. Estamos en etapa temprana y me interesa mucho la mirada de alguien de banca empresarial sobre cómo evalúan hoy los canales digitales de adquisición — charla informal de 15 minutos, sin propuesta comercial. ¿Te animas?</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>Armado</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>EXPLORATORIO — cero pitch formal a bancos (pendientes de seguridad abiertos). Mensaje listo — pendiente de envío por Jhey (no enviado)</t>
         </is>
@@ -1799,22 +1896,33 @@
           <t>CEO — Ortodoncia Funcional (ortodoncia enfocada en bruxismo y ATM), docente universitaria, Medellín</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>No capturado (corrida previa a la corrección del 3 ago)</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>CEO y dueña de su propia clínica de ortodoncia (Ortodoncia Funcional) en Medellín — perfil público de LinkedIn</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>Hola, Carolina. Vi que eres la CEO de Ortodoncia Funcional en Medellín, enfocada en bruxismo y ATM. Estoy construyendo Neggo, una plataforma que conecta negocios de salud y estética de la ciudad con clientes verificados que ya están buscando activamente su servicio — pagas solo por resultado real (CPL bajo), sin pauta ni permanencia. Los primeros 50 comercios de Medellín reciben el Sello de Confianza gratis. ¿Te cuento en 5-10 minutos cómo funciona?</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>Armado</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>Mensaje listo — pendiente de envío por Jhey (no enviado). Próxima acción: esperar a que Jhey lo envíe.</t>
         </is>
@@ -1841,22 +1949,33 @@
           <t>Co-Fundadora y Gerente General — Wellness Spa by Clínica Antienvejecimiento, Medellín</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>No capturado (corrida previa a la corrección del 3 ago)</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Co-fundadora y gerente general de su propio spa de bienestar/antienvejecimiento en Medellín — perfil público de LinkedIn</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>Hola, Lucía. Vi tu rol como co-fundadora y gerente general de Wellness Spa by Clínica Antienvejecimiento en Medellín. Estoy construyendo Neggo, una plataforma que conecta negocios de belleza y bienestar de la ciudad con clientes verificados que ya están buscando el servicio — pagas solo por resultado real (CPL bajo), sin pauta ni permanencia. Los primeros 50 comercios de Medellín obtienen el Sello de Confianza gratis. ¿Te cuento en 5-10 minutos cómo funciona?</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>Armado</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>Mensaje listo — pendiente de envío por Jhey (no enviado). Próxima acción: esperar a que Jhey lo envíe.</t>
         </is>
@@ -1883,22 +2002,33 @@
           <t>Fundador y Director General — Gimnasio Internacional de Medellín</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>No capturado (corrida previa a la corrección del 3 ago)</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Fundador y director general de su propio gimnasio en Medellín — perfil público de LinkedIn</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>Hola, Ernesto. Vi que eres fundador y director general de Gimnasio Internacional de Medellín. Estoy construyendo Neggo, una plataforma que conecta negocios de la ciudad —incluyendo gimnasios— con clientes verificados que ya están buscando membresía o servicio, pagando solo por resultado real (CPL bajo), sin pauta ni permanencia. Los primeros 50 comercios de Medellín obtienen el Sello de Confianza gratis. ¿Te cuento en 5-10 minutos cómo funciona?</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>Armado</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>Mensaje listo — pendiente de envío por Jhey (no enviado). Próxima acción: esperar a que Jhey lo envíe.</t>
         </is>
@@ -1925,22 +2055,33 @@
           <t>CEO — AGL Eventos Empresariales; Directora Ejecutiva — Asociación Antioqueña de Otorrinolaringología, Medellín</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>No capturado (corrida previa a la corrección del 3 ago)</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>CEO de su propia empresa de eventos empresariales (AGL Eventos Empresariales) en Medellín — perfil público de LinkedIn</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>Hola, Adriana. Vi que eres CEO de AGL Eventos Empresariales en Medellín. Estoy construyendo Neggo, una plataforma que conecta negocios de eventos de la ciudad con clientes verificados que ya están buscando organizar algo — pagas solo por resultado real (CPL bajo), sin pauta ni permanencia. Los primeros 50 comercios de Medellín reciben el Sello de Confianza gratis. ¿Te cuento en 5-10 minutos cómo funciona?</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>Armado</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>Mensaje listo — pendiente de envío por Jhey (no enviado). Próxima acción: esperar a que Jhey lo envíe.</t>
         </is>
@@ -1967,22 +2108,33 @@
           <t>Fundadora — Buen Provecho; Especialista en Eventos Corporativos &amp; Ferias Comerciales, Medellín</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>No capturado (corrida previa a la corrección del 3 ago)</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>Fundadora de Buen Provecho, especialista en eventos corporativos y ferias comerciales en Medellín — perfil público de LinkedIn</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>Hola, Angélica. Vi tu trabajo como fundadora de Buen Provecho y especialista en eventos corporativos y ferias comerciales en Medellín. Estoy construyendo Neggo, una plataforma que conecta negocios de eventos de la ciudad con clientes verificados que ya están buscando el servicio, pagando solo por resultado (CPL bajo), sin pauta ni permanencia. Los primeros 50 comercios de Medellín obtienen el Sello de Confianza gratis. ¿Te cuento en 5-10 minutos cómo funciona?</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
         <is>
           <t>Armado</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>Mensaje listo — pendiente de envío por Jhey (no enviado). Próxima acción: esperar a que Jhey lo envíe.</t>
         </is>

</xml_diff>

<commit_message>
docs: agregar hoja Instagram al tracker de prospección
</commit_message>
<xml_diff>
--- a/docs/tracker-prospectos-neggo.xlsx
+++ b/docs/tracker-prospectos-neggo.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospectos" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LinkedIn" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instagram" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospectos'!$A$1:$J$20</definedName>
@@ -21,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -42,6 +43,11 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="3">
@@ -69,7 +75,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -78,6 +84,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1530,7 +1537,6 @@
           <t>No capturado (corrida previa a la corrección del 3 ago)</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Fundador de agencia con clientes pyme en Medellín — perfil público de LinkedIn</t>
@@ -1583,7 +1589,6 @@
           <t>No capturado (corrida previa a la corrección del 3 ago)</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Consultor de marketing digital y mentor de emprendedores en Medellín — perfil público de LinkedIn</t>
@@ -1636,7 +1641,6 @@
           <t>No capturado (corrida previa a la corrección del 3 ago)</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
       <c r="G4" s="2" t="inlineStr">
         <is>
           <t>Implementa CRM y sistemas de ventas con WhatsApp para equipos comerciales — perfil público de LinkedIn. OJO: ciudad no confirmada</t>
@@ -1689,7 +1693,6 @@
           <t>No capturado (corrida previa a la corrección del 3 ago)</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
       <c r="G5" s="2" t="inlineStr">
         <is>
           <t>5+ años en gestión comercial inmobiliaria en Medellín — perfil público de LinkedIn</t>
@@ -1742,7 +1745,6 @@
           <t>No capturado (corrida previa a la corrección del 3 ago)</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
       <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Rol reciente de Gerente de Proyectos en promotora/constructora de Medellín — perfil público de LinkedIn</t>
@@ -1795,7 +1797,6 @@
           <t>No capturado (corrida previa a la corrección del 3 ago)</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
       <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Gerente de sucursal Bancolombia en Medellín con experiencia en banca pyme — perfil público de LinkedIn</t>
@@ -1848,7 +1849,6 @@
           <t>No capturado (corrida previa a la corrección del 3 ago)</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
       <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Gerente de Banca Empresarial en Banco de Occidente, Medellín — perfil público de LinkedIn</t>
@@ -1901,7 +1901,6 @@
           <t>No capturado (corrida previa a la corrección del 3 ago)</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
       <c r="G9" s="2" t="inlineStr">
         <is>
           <t>CEO y dueña de su propia clínica de ortodoncia (Ortodoncia Funcional) en Medellín — perfil público de LinkedIn</t>
@@ -1954,7 +1953,6 @@
           <t>No capturado (corrida previa a la corrección del 3 ago)</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
       <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Co-fundadora y gerente general de su propio spa de bienestar/antienvejecimiento en Medellín — perfil público de LinkedIn</t>
@@ -2007,7 +2005,6 @@
           <t>No capturado (corrida previa a la corrección del 3 ago)</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
       <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Fundador y director general de su propio gimnasio en Medellín — perfil público de LinkedIn</t>
@@ -2060,7 +2057,6 @@
           <t>No capturado (corrida previa a la corrección del 3 ago)</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
       <c r="G12" s="2" t="inlineStr">
         <is>
           <t>CEO de su propia empresa de eventos empresariales (AGL Eventos Empresariales) en Medellín — perfil público de LinkedIn</t>
@@ -2113,7 +2109,6 @@
           <t>No capturado (corrida previa a la corrección del 3 ago)</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
       <c r="G13" s="2" t="inlineStr">
         <is>
           <t>Fundadora de Buen Provecho, especialista en eventos corporativos y ferias comerciales en Medellín — perfil público de LinkedIn</t>
@@ -2144,4 +2139,82 @@
   <autoFilter ref="A1:H8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Tipo de perfil (Comercio directo/Conector/Banco-Constructora)</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Usuario Instagram (@)</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Nombre / Rubro</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Perfil Instagram (link)</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Bio real / gancho</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Mensaje armado</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Próxima acción</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>Estado (Armado/Enviado por Jhey)</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>Notas</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs: agregar 4 perfiles nuevos a prospección LinkedIn (corrida 3 ago)
</commit_message>
<xml_diff>
--- a/docs/tracker-prospectos-neggo.xlsx
+++ b/docs/tracker-prospectos-neggo.xlsx
@@ -1441,7 +1441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:K17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -2132,6 +2132,226 @@
       <c r="K13" s="2" t="inlineStr">
         <is>
           <t>Mensaje listo — pendiente de envío por Jhey (no enviado). Próxima acción: esperar a que Jhey lo envíe.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Conector</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Felipe Andrés Betancurt Molina</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>CMO Fraccional — iA &amp; Growth Marketing, Estratega Senior de Pauta Digital y Crecimiento (profesional independiente), Medellín</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/felipebetancurt/</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Dominique van Meerbeke Camargo</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Se presenta como "Líder de Marketing CMO (Fraccional)" con foco en growth marketing con IA y pauta digital para sus clientes — perfil público de LinkedIn</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Hola, Felipe. Tu perfil como CMO Fraccional y tu foco en growth marketing con IA me llamó la atención — es justo el tipo de mirada que necesitan las pymes de Medellín para no depender solo de pauta. Estoy construyendo Neggo: conectamos negocios locales con clientes ya verificados que buscan su servicio, cobrando solo por resultado (CPL). Para los clientes que lideras como CMO Fraccional, esto podría sumar como canal de demanda complementario a la estrategia que ya armas. ¿Vale la pena que lo conversemos un rato esta semana?</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Armado</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Mensaje listo — pendiente de envío por Jhey (no enviado).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Comercio directo</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Juan Esteban Torres Zarama</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Arquitecto, Fundador — Zarama Arquitectos (diseño y remodelación de espacios residenciales y comerciales), Envigado</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/juan-esteban-torres-zarama-239951149/</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="n"/>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Fundador de su propio estudio de arquitectura, enfocado en remodelación de espacios residenciales y comerciales con enfoque "funcional y estética, sostenible" — perfil público de LinkedIn</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Hola, Juan Esteban. Vi que desde Zarama Arquitectos trabajas remodelación de espacios residenciales y comerciales con un enfoque en arquitectura funcional y sostenible — un segmento con ticket alto y clientes que buscan confiar en quien va a intervenir su casa o local. En Neggo conectamos negocios de Medellín con clientes verificados que ya están buscando ese servicio, cobrando por resultado real y sin pauta ni contrato de permanencia. Los primeros 50 comercios de la ciudad quedan con el Sello de Confianza sin costo. ¿Te sirve que te muestre cómo funciona en una llamada corta esta semana?</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>Armado</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>Mensaje listo — pendiente de envío por Jhey (no enviado). Categoría Remodelación (sección 1 ICP) — primer perfil de esta categoría en el canal LinkedIn.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Comercio directo</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Maritza Flórez</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Dermatóloga, Co-Fundadora — Affrenchy &amp; Maritza Flórez Dermatólogo (dermo-cosmética), Área metropolitana de Medellín</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/maritza-florez-dermat%C3%B3loga/</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="n"/>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Dermatóloga y co-fundadora de su propia marca enfocada en dermo-cosmética (Affrenchy), además de su consulta propia — perfil público de LinkedIn</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Hola, Maritza. Vi que además de tu consulta dermatológica lideras Affrenchy, enfocado en dermo-cosmética — una combinación que le da a tus pacientes algo más integral que una consulta puntual. Estamos armando Neggo en Medellín para conectar negocios de salud y estética con clientes que ya están buscando activamente ese tipo de servicio, con pago solo por resultado y sin permanencia. Al ser de las primeras 50 negocios que se sumen en Medellín, el Sello de Confianza queda incluido sin costo. ¿Charlamos 10 minutos para que veas si te hace sentido?</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>Armado</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>Mensaje listo — pendiente de envío por Jhey (no enviado).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Banco-Constructora</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Manuela Restrepo Barrios</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Gerente Regional / Gerente Estructuración — Fiducia y Fideicomisos, Credicorp Capital Fiduciaria, Medellín</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/manurestrepob/</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Andrés (a confirmar si es Andrés Escobar Uribe)</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Compartió en su perfil la noticia del cambio de liderazgo/presidencia de Credicorp Capital Fiduciaria (transición tras 15+ años del anterior presidente) — actividad reciente real, perfil público de LinkedIn</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Hola, Manuela. Vi que compartiste la noticia del cambio de liderazgo en Credicorp Capital Fiduciaria — se siente distinto ver una transición así después de tantos años con el mismo liderazgo al frente. Estoy construyendo Neggo, una plataforma en Medellín que conecta clientes verificados con negocios y, más adelante, con estructuración de negocios inmobiliarios y financieros. Estamos en etapa temprana y me interesa mucho tu mirada desde estructuración y fiducia sobre cómo se evalúa hoy un canal de adquisición de clientes nuevo — sin ninguna propuesta de por medio, solo una charla de fundador a alguien que conoce el terreno. ¿Te late una charla corta esta semana, sin nada formal de por medio?</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>Armado</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>EXPLORATORIO — sin pitch formal ni CTA de registro (regla secciones 9-10). Mensaje listo — pendiente de envío por Jhey (no enviado). Verificar identidad exacta del contacto en común 'Andrés' antes de enviar.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: agregar 4 perfiles nuevos a prospección Instagram
</commit_message>
<xml_diff>
--- a/docs/tracker-prospectos-neggo.xlsx
+++ b/docs/tracker-prospectos-neggo.xlsx
@@ -2367,7 +2367,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2434,6 +2434,214 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Comercio directo</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>@almapranaspa</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Alma Prana Spa — Belleza/Spa</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/almapranaspa/</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Bio: "Spa medellin| limpieza facial|masajes | cumpleaños, aniversario, spa niñas spa holístico| despedida soltera". Calle 48 # 77-34, Medellín, Antioquia (dirección real en el perfil). Cuenta verificada, 713 mil seguidores. Gancho real: reel publicado hace 1 semana, "Súper paquete de parejas #parejas #spaparejas #regalo", en colaboración con @soyestefaniavelez.</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Hola 👋 Me encontré su reel del paquete de parejas (el de hace una semana con @soyestefaniavelez) — buenísima idea para reservas de último minuto. Soy de Neggo: llevamos clientes de Medellín que ya buscan spa para parejas o cumpleaños directo a negocios como el de ustedes, cobrando solo cuando el lead es real. Los primeros 50 comercios de la ciudad se llevan el Sello de Confianza sin costo. ¿Charlamos 5 minutos?</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Armado</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Cuenta grande (713 mil seguidores) — igual encaja en ICP Belleza/Spa Medellín, dirección confirmada en bio. Mensaje listo, pendiente de envío por Jhey (no enviado).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Comercio directo</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>@sermasfitnesscenter</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Ser+Fit Fitness Center — Gimnasio</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/sermasfitnesscenter/</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Bio: "Tu mejor versión empieza aquí. Planes personalizados - semipersonalizados, fisioterapia. Profesionales expertos, tu SALUD nos importa". Post de 30 semanas confirma dirección real: Calle 24 #44-46, Medellín. 2928 seguidores, WhatsApp real en bio. Gancho real: combinan planes personalizados/semipersonalizados con fisioterapia, no solo membresía estándar.</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Hola 👋 Vi que en Ser+Fit combinan planes personalizados con fisioterapia, no solo membresía estándar — eso diferencia bastante en Medellín. Desde Neggo conectamos gimnasios con personas que ya están buscando entrenar en su zona, y solo se paga por lead entregado, cero pauta fija. ¿Les interesa que les cuente cómo funciona? 5 minutos, sin compromiso.</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Armado</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Mensaje listo, pendiente de envío por Jhey (no enviado).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Comercio directo</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>@gamezconstruye</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Alejandro Gámez / Grupo Gámez — Remodelación</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/gamezconstruye/</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Bio: "Alejandro Gámez | Acabados y Obra — Desarrollador Inmobiliario, Estructuración · Construcción · Acabados, +40 entregas con @non_construcciones". Cuenta verificada, 12,8 mil seguidores, web grupogamez.com.co. Gancho real: post de hace 3 semanas con hashtags #AcabadosMedellin #ConstruccionAntioquia #RemodelacionMedellin, detallando un apartamento de 49 m² remodelado (revocado, estuco y pintura en 152 m²) por $7.900.000.</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Hola Alejandro 👋 Me llamó la atención el post donde desglosás el costo real de un apto de 49m² remodelado ($7.900.000, con estuco y pintura incluidos) — pocos son tan transparentes con el número. En Neggo llevamos clientes de Medellín que ya están cotizando remodelación directo a negocios como el tuyo, pago solo por resultado. ¿Vemos 5 minutos cómo encaja con lo que hacés?</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Armado</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Mensaje listo, pendiente de envío por Jhey (no enviado).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Comercio directo</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>@mels_micropigmentacion</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Melissa Cañaveral / MELS — Belleza/Estética (micropigmentación, cejas, pestañas)</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/mels_micropigmentacion/</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Bio: "Creo belleza natural y te ayudo a cumplir tus sueños. Especialista en cejas y trainer 📍Medellín". Cuenta verificada, 22,1 mil seguidores. Gancho real: post que anuncia la nueva sede en Laureles ("aquí te mostramos el paso a paso desde el Burger King del segundo parque"), servicios: micro ultranatural, hairstroke, nanobrows, extensiones de pestañas, lifting &amp; laminado.</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Hola Melissa 👋 Vi que Mels estrenó sede en Laureles, cerca del Burger King del segundo parque — felicitaciones por el crecimiento. Con Neggo conectamos negocios de belleza en Medellín con clientas que ya buscan cejas, pestañas o micropigmentación, y solo pagás cuando el lead es real. Como parte de los primeros 50 comercios, el Sello de Confianza queda gratis. ¿Te cuento en 5 minutos?</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Armado</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Mensaje listo, pendiente de envío por Jhey (no enviado).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: agregar 3 perfiles nuevos a prospección LinkedIn (4 ago, corrida 9am)
</commit_message>
<xml_diff>
--- a/docs/tracker-prospectos-neggo.xlsx
+++ b/docs/tracker-prospectos-neggo.xlsx
@@ -1441,7 +1441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:K20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -2352,6 +2352,173 @@
       <c r="K17" s="2" t="inlineStr">
         <is>
           <t>EXPLORATORIO — sin pitch formal ni CTA de registro (regla secciones 9-10). Mensaje listo — pendiente de envío por Jhey (no enviado). Verificar identidad exacta del contacto en común 'Andrés' antes de enviar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Comercio directo</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Anamaría Henao Cardona</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Periodoncista, Co-fundadora — Binnua (práctica clínica en Medellín y Rionegro)</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/anamar%C3%ADa-henao-cardona-457296103/</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="n"/>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Especialidad en periodoncia y co-fundadora de Binnua, con consulta activa en dos ciudades (Medellín y Rionegro) — dato del titular de su perfil público de LinkedIn</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Hola, Anamaría. Vi que además de tu práctica en periodoncia llevas Binnua con presencia en Medellín y Rionegro — sostener dos sedes no es poca cosa. Estamos construyendo Neggo en Medellín: conectamos negocios de salud y estética con pacientes que ya están buscando el servicio, cobrando solo por resultado real (CPL bajo), sin pauta genérica ni contrato de permanencia. Si te sumas entre los primeros 50 comercios de la ciudad, el Sello de Confianza queda incluido sin costo. ¿Vale la pena que te muestre cómo funciona en una llamada de 10 minutos?</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Armado</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>Categoría Salud/Estética (ICP sección 1). Mensaje listo — pendiente de envío por Jhey (no enviado).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Banco-Constructora</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Carolina Zuleta</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Gerente Comercial y Desarrollo de Negocios — Constructora Convel, Medellín</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/carolina-zuleta/</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Andrés (a confirmar si es Andrés Escobar Uribe)</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Post reciente (hace ~1 mes) sobre Casa Nua Country, proyecto de Constructora Convel diseñado para calidad de vida de adultos mayores con foco en accesibilidad e integración social — actividad real de su perfil público de LinkedIn</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Hola, Carolina. Vi tu post sobre Casa Nua Country, el proyecto de Constructora Convel pensado para la calidad de vida de los adultos mayores — el foco en accesibilidad e integración social no es el ángulo típico de un desarrollo inmobiliario. Estoy construyendo Neggo, una plataforma en Medellín que conecta clientes verificados con negocios y, más adelante, con estructuración de proyectos inmobiliarios. Estamos en etapa temprana y me interesaría mucho tu mirada desde desarrollo de negocios sobre cómo llegan hoy los leads a un proyecto así — sin ninguna propuesta comercial de por medio, solo aprender de alguien que vive el sector. ¿Te animas a un café virtual de 15 minutos esta semana?</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Armado</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>EXPLORATORIO — sin pitch formal ni CTA de registro (regla secciones 9-10). Verificar identidad exacta del contacto en común 'Andrés' antes de enviar. Mensaje listo — pendiente de envío por Jhey (no enviado).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Conector</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Mario Raguá Rueda</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Mentor de pymes, Fundador — ivestinGO (programa Ruta Financiera / Signos Vitales del Negocio), Colombia</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/carlos-mario-ragu%C3%A1-rueda-b682b7170/</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Carlos Guayara, Esteban Penaloza Guzmán</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Programa activo 'Ruta Financiera' en ivestinGO, ayudando a dueños de pyme a fortalecer su estructura financiera para atraer inversionistas — publicaciones recientes reales en su perfil de LinkedIn</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Hola, Carlos Mario. Vi tu programa Ruta Financiera en ivestinGO, ayudando a dueños de pyme a fortalecer su estructura financiera para verse atractivos ante un inversionista — un ángulo que pocos mentores tocan tan directo. Estoy construyendo Neggo: conectamos negocios de Medellín con clientes ya verificados y con score financiero visible, cobrando solo por resultado. Varias de las pymes que acompañas en Signos Vitales del Negocio podrían encajar como el tipo de negocio que necesita ese canal de demanda, sin tener que pautar. ¿Te interesa que lo charlemos 10 minutos para ver si hay sinergia real entre lo que hacen ustedes y lo que estamos construyendo?</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>Armado</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>Mensaje listo — pendiente de envío por Jhey (no enviado).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: reescribir 3 mensajes de Instagram con tono profesional + gancho Neggo Ads
</commit_message>
<xml_diff>
--- a/docs/tracker-prospectos-neggo.xlsx
+++ b/docs/tracker-prospectos-neggo.xlsx
@@ -2637,7 +2637,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Hola 👋 Vi que en Ser+Fit combinan planes personalizados con fisioterapia, no solo membresía estándar — eso diferencia bastante en Medellín. Desde Neggo conectamos gimnasios con personas que ya están buscando entrenar en su zona, y solo se paga por lead entregado, cero pauta fija. ¿Les interesa que les cuente cómo funciona? 5 minutos, sin compromiso.</t>
+          <t>Hola Ser+Fit. Vi que combinan planes personalizados con fisioterapia — no es la propuesta genérica de la mayoría de gimnasios en Medellín, y se nota que ya tienen una base sólida de clientes. Estoy construyendo Neggo: conectamos negocios como el suyo con personas que ya buscan entrenar en su zona, con score financiero verificado, y cobramos solo cuando el lead es real — no compite con lo que ya hacen, lo complementa. Además estamos armando Neggo Ads, para que los comercios aliados también puedan gestionar su pauta en Meta/Google desde la misma plataforma; si les interesa quedar entre los primeros en probarlo, se los aviso apenas esté listo. ¿Hablamos 10 minutos?</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -2647,12 +2647,12 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>No lo envio por que siento que no damos valor por ahora.</t>
+          <t>Armado</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Mensaje listo, pendiente de envío por Jhey (no enviado).</t>
+          <t>Mensaje listo, pendiente de envío por Jhey (no enviado). | Reescrito 4 ago: tono más profesional para cuenta grande/consolidada + mención honesta de Neggo Ads (ver sección 6.1 de la estrategia). Mensaje listo — pendiente de envío por Jhey (no enviado).</t>
         </is>
       </c>
     </row>
@@ -2689,7 +2689,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Hola Alejandro 👋 Me llamó la atención el post donde desglosás el costo real de un apto de 49m² remodelado ($7.900.000, con estuco y pintura incluidos) — pocos son tan transparentes con el número. En Neggo llevamos clientes de Medellín que ya están cotizando remodelación directo a negocios como el tuyo, pago solo por resultado. ¿Vemos 5 minutos cómo encaja con lo que hacés?</t>
+          <t>Hola Alejandro. El post donde desglosás el costo real de un apartamento remodelado ($7.900.000, con el detalle de estuco y pintura) es del tipo de transparencia que no se ve seguido en el sector — y con más de 40 entregas y equipo propio, Grupo Gámez ya tiene una trayectoria que habla sola. Estoy construyendo Neggo: llevamos clientes de Medellín que ya están cotizando remodelación directo a negocios serios, con score financiero verificado y pago solo por resultado — no reemplaza lo que ya construyeron, filtra la demanda que ya está lista para contratar. A futuro también van a poder gestionar pauta en Meta/Google desde la misma plataforma con Neggo Ads, hoy en construcción. ¿Vemos 10 minutos cómo encaja con lo que hacen?</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -2699,12 +2699,12 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>No lo envio por que siento que no damos valor por ahora.</t>
+          <t>Armado</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Mensaje listo, pendiente de envío por Jhey (no enviado).</t>
+          <t>Mensaje listo, pendiente de envío por Jhey (no enviado). | Reescrito 4 ago: tono más profesional para cuenta grande/consolidada + mención honesta de Neggo Ads (ver sección 6.1 de la estrategia). Mensaje listo — pendiente de envío por Jhey (no enviado).</t>
         </is>
       </c>
     </row>
@@ -2741,7 +2741,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Hola Melissa 👋 Vi que Mels estrenó sede en Laureles, cerca del Burger King del segundo parque — felicitaciones por el crecimiento. Con Neggo conectamos negocios de belleza en Medellín con clientas que ya buscan cejas, pestañas o micropigmentación, y solo pagás cuando el lead es real. Como parte de los primeros 50 comercios, el Sello de Confianza queda gratis. ¿Te cuento en 5 minutos?</t>
+          <t>Hola Melissa. Felicitaciones por la nueva sede en Laureles — con más de 22 mil seguidores y una cuenta verificada, MELS ya tiene el reconocimiento que a la mayoría le cuesta años lograr. Estoy construyendo Neggo: conectamos negocios de belleza en Medellín con clientas que ya buscan cejas, pestañas o micropigmentación y llegan con score financiero verificado — el objetivo no es reemplazar el trabajo de marca que ya hicieron, sino entregarles la demanda que ya está lista para agendar. Como parte de los primeros 50 comercios, el Sello de Confianza (verificación real del negocio, no solo un ícono) queda sin costo. También estamos construyendo Neggo Ads para gestionar pauta en Meta/Google desde la misma plataforma — si te interesa quedar en la lista de espera, te aviso apenas esté listo. ¿Te cuento en 10 minutos?</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -2751,12 +2751,12 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>No lo envio por que siento que no damos valor por ahora.</t>
+          <t>Armado</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Mensaje listo, pendiente de envío por Jhey (no enviado).</t>
+          <t>Mensaje listo, pendiente de envío por Jhey (no enviado). | Reescrito 4 ago: tono más profesional para cuenta grande/consolidada + mención honesta de Neggo Ads (ver sección 6.1 de la estrategia). Mensaje listo — pendiente de envío por Jhey (no enviado).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: agregar 5 perfiles nuevos a prospección LinkedIn (4 ago, corrida automática)
</commit_message>
<xml_diff>
--- a/docs/tracker-prospectos-neggo.xlsx
+++ b/docs/tracker-prospectos-neggo.xlsx
@@ -1580,7 +1580,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:K22"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -2490,6 +2490,279 @@
       <c r="K17" s="2" t="inlineStr">
         <is>
           <t>EXPLORATORIO — sin pitch formal ni CTA de registro (regla secciones 9-10). Mensaje listo — pendiente de envío por Jhey (no enviado). Verificar identidad exacta del contacto en común 'Andrés' antes de enviar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="352" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Comercio directo</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Silviana Cardona</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Fundadora y Gerente — Viajes Destino Antioquia (agencia de viajes con enfoque en experiencias de impacto territorial), Colombia</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/silviana-cardona-03969540/</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="n"/>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Fundadora de su propia agencia de viajes (Viajes Destino Antioquia), enfocada en "experiencias con propósito, impacto territorial y valor estratégico" y no en turismo genérico — perfil público de LinkedIn</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Hola, Silviana. Vi que desde Viajes Destino Antioquia diseñas experiencias con impacto territorial, no solo paquetes genéricos — eso ya dice bastante sobre cómo trabajas. Estoy armando Neggo, una plataforma en Medellín que conecta negocios como el tuyo con clientes que ya están buscando activamente el servicio, cobrando solo cuando el contacto es real. Cada comercio que entra lo verificamos antes de listarlo, así el cliente sabe que está hablando con una agencia de verdad. Sin pauta, sin permanencia, y los primeros 50 comercios de Medellín quedan con el Sello de Confianza sin costo. ¿Te cuento cómo funciona en una llamada corta?</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Armado</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>Mensaje listo — pendiente de envío por Jhey (no enviado). Categoría: Viaje — primer perfil de esta categoría en el canal LinkedIn (tenía cero prospectos previos en el tracker).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="358" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Comercio directo</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Alvaro Aguirre</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Arquitecto, Fundador y Gerente General — Gatitud® SAS (muebles y accesorios ecoamigables para gatos), Medellín</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/alvaro-aguirre-85172255/</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="n"/>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Arquitecto con +13 años en diseño de producto sostenible, fundador de su propia marca de muebles para gatos (Gatitud®) — publica casi a diario sobre sus productos (torres, rascadores de cartón, hamacas) con marca y fotografía propias, perfil público de LinkedIn</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Hola, Álvaro. Llevo un rato viendo tus publicaciones de Gatitud — la torre y los rascadores de cartón se ven bien pensados, se nota el trasfondo de arquitecto detrás del diseño. Con Neggo conectamos negocios de Medellín con clientes que ya buscan ese tipo de producto, y solo cobramos cuando el contacto es real, sin necesidad de pautar. Trabajamos con código anti-phishing en cada conversación, para que quien te escriba sepa que el mensaje viene realmente de nosotros. Los primeros 50 comercios de la ciudad reciben el Sello de Confianza sin costo. ¿Vale la pena que hablemos 10 minutos?</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Armado</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>Mensaje listo — pendiente de envío por Jhey (no enviado). Categoría: Mascotas — primer perfil de esta categoría en el canal LinkedIn (tenía cero prospectos previos en el tracker).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="376" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Comercio directo</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Andrea Muñoz Agudelo</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Fashion Designer &amp; Stylist, Fundadora — Brisa Morena Swimwear, Área metropolitana de Medellín</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/andreamunoza/</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="n"/>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Fundadora de su propia marca de trajes de baño (Brisa Morena) y además especialista en escaparatismo y decoración de tiendas — perfil público de LinkedIn</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Hola, Andrea. Vi que además de diseñar para Brisa Morena manejas escaparatismo y decoración de tiendas — un ojo que pocas marcas de moda en Medellín tienen tan desarrollado. Estoy construyendo Neggo, una plataforma que conecta negocios de moda y accesorios con clientes que ya están buscando comprar, cobrando por resultado real y sin contrato de permanencia. Cumplimos la Ley 1581 de protección de datos, así que tanto tu marca como tus clientes quedan cubiertos. Como parte de los primeros 50 comercios de la ciudad, te llevas el Sello de Confianza gratis. ¿Te cuento los detalles en una llamada corta esta semana?</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>Armado</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>Mensaje listo — pendiente de envío por Jhey (no enviado). Categoría: Moda y Accesorios — primer perfil de esta categoría en el canal LinkedIn (tenía cero prospectos previos en el tracker).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="324" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Conector</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Michael Andrés García Pérez</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Consultor Empresarial | Director Comercial | Estrategia Comercial y Análisis Financiero | 20 años asesorando pymes, Medellín</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/michael-andr%C3%A9s-garc%C3%ADa-p%C3%A9rez-1aa56252/</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Daniel (contacto en común — apellido no confirmado en la búsqueda)</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Publicó hace 3 días sobre el error de confundir "vender más" con "ganar más" y la importancia de estructurar el plan de cuentas y proyectar flujo de caja a 12 meses — consultor activo asesorando pymes y empresarios en Medellín, perfil público de LinkedIn</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Hola, Michael. Leí tu publicación sobre confundir vender más con ganar más — la parte de estructurar bien el plan de cuentas antes de proyectar flujo de caja es justo la disciplina que le falta a muchos comercios que estoy conociendo en Medellín. Estoy construyendo Neggo: conectamos negocios locales con clientes verificados que ya buscan su servicio, cobrando solo por resultado. Varios de los empresarios que asesoras podrían necesitar justo ese canal de demanda, sin gastar en pauta que no controlan. ¿Te interesa que lo conversemos, aunque sea para que me des tu mirada de consultor?</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>Armado</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>Mensaje listo — pendiente de envío por Jhey (no enviado). Contacto en común 'Daniel' sin apellido confirmado en la búsqueda — verificar identidad antes de enviar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="714" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Banco-Constructora</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Jorge Montoya Tobón</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Gerente Comercial — Latam Trade Capital (factoring / financiamiento empresarial), Medellín</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/jorge-montoya-tob%C3%B3n-904351147/</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Angela y Esteban Penaloza Guzmán (2 contactos en común, según LinkedIn)</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Su empresa (Latam Trade Capital) compartió hace 1 semana contenido sobre factoring como alternativa de liquidez y su participación reciente en FinteChile — perfil verificado, activo en el ecosistema fintech regional, perfil público de LinkedIn</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Hola, Jorge. Vi que tenemos contactos en común (Esteban, entre otros) y que en Latam Trade Capital han estado compartiendo bastante sobre factoring como alternativa de liquidez — hace poco fueron parte de FinteChile, se nota que el equipo está metido de lleno en el ecosistema fintech de la región. Estoy construyendo Neggo, una plataforma en Medellín que conecta clientes verificados con negocios y, más adelante, con financiamiento. Estamos en etapa temprana, y me interesa tu mirada desde banca pyme y fintech sobre cómo se evalúa hoy un canal de adquisición nuevo — sin ninguna propuesta formal de por medio, solo una charla de fundador a alguien que vive el sector. ¿Tienes 15 minutos esta semana para un café virtual?</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>Armado</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>EXPLORATORIO — sin pitch formal ni CTA de registro (regla secciones 9-10, sector fintech/factoring adyacente a banca). Cuenta verificada, 2.236 seguidores — no cumple el umbral de 'cuenta grande' de la sección 6.1 (esa sección aplica al pitch de comercios directos, no a este segmento exploratorio). Mensaje listo — pendiente de envío por Jhey (no enviado).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: agregar 3 perfiles nuevos a prospección Instagram (Mascotas, Muebles, Moda)
</commit_message>
<xml_diff>
--- a/docs/tracker-prospectos-neggo.xlsx
+++ b/docs/tracker-prospectos-neggo.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -76,6 +76,10 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -109,7 +113,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -133,6 +137,9 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2778,7 +2785,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="10.1640625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -3261,6 +3268,162 @@
         </is>
       </c>
     </row>
+    <row r="10" ht="126" customHeight="1">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>Comercio directo</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>@orejitas_exoticas</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>Orejitas Exótica — Mascotas (hábitats y alimentos para conejos, cobayas, hamsters, erizos)</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/orejitas_exoticas/</t>
+        </is>
+      </c>
+      <c r="F10" s="10" t="inlineStr">
+        <is>
+          <t>Bio: "hábitats y alimentos para conejos|cobayas|hamsters|erizos|ratas". "TIENDA VIRTUAL", "NO VENDEMOS ANIMALES", "NO LLAMADAS". Dirección real: Calle 49#38-43 boulevard 49, Medellín, Antioquia. 6.620 seguidores, 369 publicaciones, cuenta activa desde 2021 con posteo consistente. Gancho real: post de hace 13 semanas (4 de mayo) sobre una "Esfera de mimbre rellena de heno y flores aromáticas" para el desgaste dental, producto 100% natural, diámetro 17cm.</t>
+        </is>
+      </c>
+      <c r="G10" s="10" t="inlineStr">
+        <is>
+          <t>Hola equipo de Orejitas Exótica. La esfera de mimbre rellena de heno que sacaron en mayo (pensada para el desgaste dental, 100% natural) es el tipo de detalle que explica por qué ya suman más de 6.600 seguidores en un nicho tan específico. Estoy construyendo Neggo: llevamos personas de Medellín que ya buscan insumos para mascotas exóticas directo a negocios serios, con score financiero verificado — no compite con la marca que ya construyeron, filtra la demanda que ya está lista para comprar. Verificamos cada comercio antes de listarlo, así que el cliente llega con confianza real, no solo con una promesa. También estamos armando Neggo Ads para gestionar pauta en Meta/Google desde la misma plataforma — si les interesa la lista de espera, aviso apenas esté listo. ¿Hablamos 10 minutos?</t>
+        </is>
+      </c>
+      <c r="H10" s="10" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="I10" s="10" t="inlineStr">
+        <is>
+          <t>Armado</t>
+        </is>
+      </c>
+      <c r="J10" s="10" t="inlineStr">
+        <is>
+          <t>Categoría: Mascotas. Cuenta grande/consolidada (6.620 seguidores, actividad consistente desde 2021) — tratamiento sección 6.1 aplicado (tono profesional, sin emoji de saludo, reconocimiento explícito antes del pitch, mención honesta de Neggo Ads en modo lista de espera). Mensaje listo, pendiente de envío por Jhey (no enviado).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="126" customHeight="1">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>Comercio directo</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>@mueblesbika</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>Muebles Bika — Muebles y Decoración (fábrica propia, hogar y oficina)</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/mueblesbika/</t>
+        </is>
+      </c>
+      <c r="F11" s="10" t="inlineStr">
+        <is>
+          <t>Bio: "Muebles modernos en Medellín. Hogar · Oficina · Diseño a medida. Fabricamos, entregamos e instalamos." 14,2 mil seguidores, 565 publicaciones. Sede confirmada en highlight "Contacto": Calle 33 # 75c-109, Laureles, Medellín, con diseñador de espacios Sergio Cardona. Gancho real: posts de junio (8 sem) "Fabricamos lo que ves. Desde 1992" y silla ergonómica "Gary" con soporte lumbar para home office, envíos a Medellín/Bogotá/Colombia, pago a cuotas con Addi.</t>
+        </is>
+      </c>
+      <c r="G11" s="10" t="inlineStr">
+        <is>
+          <t>Hola equipo de Bika. Que sigan fabricando en Medellín desde 1992 y hoy tengan diseñador propio como Sergio Cardona en la sede de Laureles dice mucho — no muchas marcas de muebles llegan a esa trayectoria sin perder calidad. Estoy construyendo Neggo: conectamos negocios de muebles y remodelación con clientes de Medellín que ya están cotizando, con score financiero verificado antes de llegarles — no reemplaza la fábrica que ya construyeron, filtra la demanda que ya está lista para comprar. Cumplimos la Ley 1581 de protección de datos, así que el cliente llega tranquilo desde el primer contacto. También estamos construyendo Neggo Ads, para pautar en Meta/Google desde la misma plataforma — si les interesa la lista de espera para cuando esté listo, aviso. ¿Vemos 10 minutos cómo encaja con lo que ya hacen?</t>
+        </is>
+      </c>
+      <c r="H11" s="10" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="I11" s="10" t="inlineStr">
+        <is>
+          <t>Armado</t>
+        </is>
+      </c>
+      <c r="J11" s="10" t="inlineStr">
+        <is>
+          <t>Categoría: Muebles y Decoración. Cuenta grande/consolidada (14.200 seguidores, fábrica propia desde 1992, sede física en Laureles, diseñador propio) — tratamiento sección 6.1 aplicado (tono profesional, sin emoji de saludo, reconocimiento explícito antes del pitch, mención honesta de Neggo Ads en modo lista de espera). Mensaje listo, pendiente de envío por Jhey (no enviado).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="126" customHeight="1">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>Comercio directo</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>@kim_boutique_medellin</t>
+        </is>
+      </c>
+      <c r="D12" s="10" t="inlineStr">
+        <is>
+          <t>Kim Boutique Medellín — Moda y Accesorios (ropa mujer, americana, al por mayor)</t>
+        </is>
+      </c>
+      <c r="E12" s="10" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/kim_boutique_medellin/</t>
+        </is>
+      </c>
+      <c r="F12" s="10" t="inlineStr">
+        <is>
+          <t>Bio: "KIM BOUTIQUE MEDELLIN | ROPA MUJER | AMERICANA. Boutique. Emprende con nosotras al por mayor. Tienda virtual. Medellín." 4.724 seguidores, 3.961 publicaciones (cuenta muy activa, varias publicaciones diarias). Gancho real: post publicado hace 6 horas, ubicación etiquetada "Poblado - Medellín", texto "Hay días en los que una se convence solita... Me lo merezco / Me encanta / ¡Me lo compro!".</t>
+        </is>
+      </c>
+      <c r="G12" s="10" t="inlineStr">
+        <is>
+          <t>Hola 👋 Vi el post de hace unas horas del "me lo merezco, me encanta, me lo compro" — buen gancho para las que dudan antes de comprar. Desde Neggo conectamos negocios de moda en Medellín con clientas que ya están buscando qué comprar, y solo cobramos cuando el lead es real, sin pauta fija. Los primeros 50 comercios se llevan el Sello de Confianza gratis (verificamos cada negocio antes de listarlo). ¿Te cuento en 5 minutos cómo funciona?</t>
+        </is>
+      </c>
+      <c r="H12" s="10" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="I12" s="10" t="inlineStr">
+        <is>
+          <t>Armado</t>
+        </is>
+      </c>
+      <c r="J12" s="10" t="inlineStr">
+        <is>
+          <t>Categoría: Moda y Accesorios. Cuenta activa y real (4.724 seguidores, 3.961 publicaciones), bajo el umbral de cuenta grande — tono casual estándar. Mensaje listo, pendiente de envío por Jhey (no enviado).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId1"/>

</xml_diff>

<commit_message>
fix: reparar columna Respuesta sugerida (Ventas) en hoja Prospectos — eliminar columna huérfana sin encabezado
</commit_message>
<xml_diff>
--- a/docs/tracker-prospectos-neggo.xlsx
+++ b/docs/tracker-prospectos-neggo.xlsx
@@ -565,10 +565,15 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t>Respuesta sugerida (Ventas)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>Fecha próxima acción</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Notas</t>
         </is>
@@ -615,12 +620,12 @@
           <t>Mensaje enviado</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-03</t>
-        </is>
-      </c>
       <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>TICKET ALTO — candidato a CPL superior a $30.000, proponerlo en la llamada. Mensaje listo — pendiente de envío por Jhey (no enviado)</t>
         </is>
@@ -667,12 +672,12 @@
           <t>Mensaje enviado</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-03</t>
-        </is>
-      </c>
       <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>TICKET ALTO — candidato a CPL superior. Mensaje listo — pendiente de envío por Jhey (no enviado)</t>
         </is>
@@ -719,12 +724,12 @@
           <t>Mensaje enviado</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-03</t>
-        </is>
-      </c>
       <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>TICKET ALTO — candidato a CPL superior. Mensaje listo — pendiente de envío por Jhey (no enviado)</t>
         </is>
@@ -771,12 +776,12 @@
           <t>Mensaje enviado</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-03</t>
-        </is>
-      </c>
       <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>TICKET ALTO — candidato a CPL superior. Mensaje listo — pendiente de envío por Jhey (no enviado)</t>
         </is>
@@ -826,19 +831,19 @@
 Allí podrán revisar tu propuesta con más detalle. ¡Gracias nuevamente!</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>CANAL: correo a mariana.valencia@cliniq.co (pidieron propuesta formal, no WhatsApp). Asunto: Propuesta Neggo — leads verificados para Cliniq. Hola Mariana, gracias por la respuesta. En Neggo vemos seguido que muchas personas posponen un procedimiento estético por miedo a caer con un negocio poco confiable — es un freno de conversión real, no solo falta de interés. Nosotros resolvemos justo eso: verificamos cada clínica antes de listarla y le garantizamos al cliente que quien lo contacta es realmente Cliniq, con Sello de Confianza y código anti-phishing. El resultado para ustedes es demanda ya calificada y con más disposición a agendar, pago solo por resultado (CPL), sin pauta fija ni permanencia. Dado el volumen y posicionamiento de Cliniq, podemos definir un CPL ajustado a ticket alto. ¿Tienen 10-15 minutos esta semana para una demo con el equipo comercial?</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>TICKET ALTO — candidato a CPL superior. Mensaje listo — pendiente de envío por Jhey (no enviado)</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> | Reescrito 4 ago con fórmula miedo-real+solución (ver marketing-neggo.md sección 9).</t>
+          <t>2026-08-04 — responder ya (ver Respuesta sugerida)</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>TICKET ALTO — candidato a CPL superior. Mensaje listo — pendiente de envío por Jhey (no enviado) | RESPONDIÓ (04 ago) — gestiona Ventas/Closer. Respuesta sugerida lista. Pendiente de que Jhey la revise y envíe.</t>
         </is>
       </c>
     </row>
@@ -883,12 +888,12 @@
           <t>Mensaje enviado</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-03</t>
-        </is>
-      </c>
       <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>TICKET ALTO. Gancho aún genérico — abrir IG y citar un post real antes de enviar. Mensaje listo — pendiente de envío por Jhey (no enviado)</t>
         </is>
@@ -937,19 +942,19 @@
 https://wa.me/573137679683</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>CANAL: WhatsApp +57 313 767 9683 (el que ellos dieron). Hola, les escribí por Instagram sobre Neggo. Muchas personas posponen un procedimiento estético por desconfianza de negocios que no conocen bien — en Neggo resolvemos eso verificando cada negocio antes de listarlo, así el cliente llega con más confianza y ya decidido. Con los 15+ años de trayectoria de Bioforma, esto suma demanda calificada adicional, pago solo por resultado (CPL), sin pauta fija. ¿Tienen 10 minutos esta semana para que les cuente cómo funciona?</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>TICKET ALTO — candidato a CPL superior. Mensaje listo — pendiente de envío por Jhey (no enviado)</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> | Reescrito 4 ago con fórmula miedo-real+solución (ver marketing-neggo.md sección 9).</t>
+          <t>2026-08-04 — responder ya (ver Respuesta sugerida)</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>TICKET ALTO — candidato a CPL superior. Mensaje listo — pendiente de envío por Jhey (no enviado) | RESPONDIÓ (04 ago) — gestiona Ventas/Closer. Respuesta sugerida lista. Pendiente de que Jhey la revise y envíe.</t>
         </is>
       </c>
     </row>
@@ -994,12 +999,12 @@
           <t>Mensaje enviado</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-03</t>
-        </is>
-      </c>
       <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>Mensaje listo — pendiente de envío por Jhey (no enviado)</t>
         </is>
@@ -1046,19 +1051,19 @@
           <t>Buen día Neggo, gracias por su interés en Clínica Láser de Piel. Por favor envíenos su portafolio a info@clinicalaserdepiel.com.co para remitirlo al área encargada, quienes en caso de estar interesados se comunicarán con usted. ¡Feliz día!</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>CANAL: correo a info@clinicalaserdepiel.com.co (pidieron "portafolio"). Asunto: Propuesta Neggo — leads verificados para Clínica Láser de Piel. Hola, gracias por la respuesta. En Neggo conectamos negocios de salud/estética en Medellín con clientes que ya buscan el servicio — muchos dejan de agendar por miedo a caer con un negocio poco confiable, y nosotros resolvemos justo eso verificando cada negocio antes de listarlo. No tengo un portafolio tradicional porque es un producto digital, pero con gusto agendo una llamada de 10-15 min para mostrarles cómo funciona en vivo, o les paso el link para que lo vean ustedes mismos. ¿Qué les sirve más?</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Mensaje listo — pendiente de envío por Jhey (no enviado)</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> | Reescrito 4 ago con fórmula miedo-real+solución (ver marketing-neggo.md sección 9).</t>
+          <t>2026-08-04 — responder ya (ver Respuesta sugerida)</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>Mensaje listo — pendiente de envío por Jhey (no enviado) | RESPONDIÓ (04 ago) — gestiona Ventas/Closer. Respuesta sugerida lista. Pendiente de que Jhey la revise y envíe.</t>
         </is>
       </c>
     </row>
@@ -1099,12 +1104,12 @@
         </is>
       </c>
       <c r="H11" s="2" t="n"/>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-03</t>
-        </is>
-      </c>
       <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>Mensaje listo — pendiente de envío por Jhey (no enviado)</t>
         </is>
@@ -1151,12 +1156,12 @@
           <t>Mensaje enviado</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-03</t>
-        </is>
-      </c>
       <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>Gancho por reforzar con un proyecto/post concreto antes de enviar. Mensaje listo — pendiente de envío por Jhey (no enviado)</t>
         </is>
@@ -1199,12 +1204,12 @@
         </is>
       </c>
       <c r="H13" s="2" t="n"/>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-03</t>
-        </is>
-      </c>
       <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>Mensaje listo — pendiente de envío por Jhey (no enviado)</t>
         </is>
@@ -1247,12 +1252,12 @@
         </is>
       </c>
       <c r="H14" s="2" t="n"/>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-03</t>
-        </is>
-      </c>
       <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
         <is>
           <t>Mensaje listo — pendiente de envío por Jhey (no enviado)</t>
         </is>
@@ -1299,12 +1304,12 @@
           <t>Mensaje enviado</t>
         </is>
       </c>
-      <c r="I15" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-03</t>
-        </is>
-      </c>
       <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
         <is>
           <t>Mensaje listo — pendiente de envío por Jhey (no enviado)</t>
         </is>
@@ -1351,19 +1356,19 @@
           <t>Hola, bienvenido a Amatsu spa, puedes comunicarte con nosotros a traves del whatsApp 3186506537 para hacer tus consultas y reserva.o si desea le responderemos por aca, mas tarde, Gracias por preferirnos.</t>
         </is>
       </c>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="I16" t="inlineStr">
         <is>
           <t>CANAL: WhatsApp 318 650 6537 (el que ellos dieron). OJO: su respuesta trató el mensaje como si Jhey quisiera reservar un servicio — aclarar primero que es una propuesta de negocio. Hola, gracias por responder. Aclarando: no busco reservar un servicio — les escribo porque estoy construyendo Neggo. Muchas personas dejan de comprar por desconfianza de negocios que no conocen; nosotros verificamos cada negocio antes de listarlo para que la clienta llegue ya con confianza. Pagan solo si el lead es real, sin pauta fija. ¿Tienen 5-10 minutos para que les cuente cómo funciona?</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>Mensaje listo — pendiente de envío por Jhey (no enviado)</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> | Reescrito 4 ago con fórmula miedo-real+solución (ver marketing-neggo.md sección 9).</t>
+          <t>2026-08-04 — responder ya (ver Respuesta sugerida)</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>Mensaje listo — pendiente de envío por Jhey (no enviado) | RESPONDIÓ (04 ago) — gestiona Ventas/Closer. Respuesta sugerida lista. Pendiente de que Jhey la revise y envíe.</t>
         </is>
       </c>
     </row>
@@ -1408,12 +1413,12 @@
           <t>No se envia por que siento que no tenemos como agregarle valor.</t>
         </is>
       </c>
-      <c r="I17" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-03</t>
-        </is>
-      </c>
       <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
         <is>
           <t>Mensaje listo — pendiente de envío por Jhey (no enviado)</t>
         </is>
@@ -1460,12 +1465,12 @@
           <t>No se envia por que siento que no tenemos como agregarle valor.</t>
         </is>
       </c>
-      <c r="I18" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-03</t>
-        </is>
-      </c>
       <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
         <is>
           <t>Mensaje listo — pendiente de envío por Jhey (no enviado)</t>
         </is>
@@ -1512,12 +1517,12 @@
           <t>No se envia por que siento que no tenemos como agregarle valor.</t>
         </is>
       </c>
-      <c r="I19" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-03</t>
-        </is>
-      </c>
       <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
         <is>
           <t>Mensaje listo — pendiente de envío por Jhey (no enviado)</t>
         </is>
@@ -1564,12 +1569,12 @@
           <t>No se envia por que siento que no tenemos como agregarle valor.</t>
         </is>
       </c>
-      <c r="I20" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-03</t>
-        </is>
-      </c>
       <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
         <is>
           <t>Mensaje listo — pendiente de envío por Jhey (no enviado)</t>
         </is>

</xml_diff>

<commit_message>
feat: portafolio B2B (PDF) + guion de demo + kit de ventas como responsabilidad permanente de Contenido/Marca (a pedido de Jhey, 4 ago)
</commit_message>
<xml_diff>
--- a/docs/tracker-prospectos-neggo.xlsx
+++ b/docs/tracker-prospectos-neggo.xlsx
@@ -1053,7 +1053,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>CANAL: correo a info@clinicalaserdepiel.com.co (pidieron "portafolio"). Asunto: Propuesta Neggo — leads verificados para Clínica Láser de Piel. Hola, gracias por la respuesta. En Neggo conectamos negocios de salud/estética en Medellín con clientes que ya buscan el servicio — muchos dejan de agendar por miedo a caer con un negocio poco confiable, y nosotros resolvemos justo eso verificando cada negocio antes de listarlo. No tengo un portafolio tradicional porque es un producto digital, pero con gusto agendo una llamada de 10-15 min para mostrarles cómo funciona en vivo, o les paso el link para que lo vean ustedes mismos. ¿Qué les sirve más?</t>
+          <t>CANAL: correo a info@clinicalaserdepiel.com.co (pidieron "portafolio"). Asunto: Propuesta Neggo — leads verificados para Clínica Láser de Piel. Hola, gracias por la respuesta. Les adjunto el portafolio de Neggo: en él vemos seguido que muchas personas posponen un procedimiento por miedo a caer con un negocio poco confiable — es un freno de conversión real. Nosotros resolvemos justo eso verificando cada negocio antes de listarlo, con Sello de Confianza y código anti-phishing, y solo cobramos por resultado (CPL), sin pauta fija. Adjunto también el detalle de cómo funciona. ¿Tienen 10-15 minutos esta semana para una demo? [Adjuntar docs/marca-assets/portafolio-neggo-b2b.pdf]</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -1063,7 +1063,7 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>Mensaje listo — pendiente de envío por Jhey (no enviado) | RESPONDIÓ (04 ago) — gestiona Ventas/Closer. Respuesta sugerida lista. Pendiente de que Jhey la revise y envíe.</t>
+          <t>Mensaje listo — pendiente de envío por Jhey (no enviado) | RESPONDIÓ (04 ago) — gestiona Ventas/Closer. Respuesta sugerida lista. Pendiente de que Jhey la revise y envíe. | Portafolio B2B real ya disponible (docs/marca-assets/portafolio-neggo-b2b.pdf), agregado a la respuesta 4 ago.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: agregar 3 perfiles nuevos a prospeccion LinkedIn (Moto, Conector, Constructora)
</commit_message>
<xml_diff>
--- a/docs/tracker-prospectos-neggo.xlsx
+++ b/docs/tracker-prospectos-neggo.xlsx
@@ -1592,7 +1592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K25"/>
+  <dimension ref="A1:K28"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -2937,6 +2937,184 @@
       <c r="K25" s="2" t="inlineStr">
         <is>
           <t>EXPLORATORIO — sin pitch formal ni CTA de registro (regla secciones 9-10, Corporación Interactuar es entidad de desarrollo/crédito pyme, adyacente a banca). Mensaje listo — pendiente de envío por Jhey (no enviado).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="400" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Comercio directo</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>David Vega Quiceno</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Gerente de Mercadeo — FP Moto, Guarne / Área metropolitana de Medellín</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/davidvega-fp-marketingmotos/</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Sebastian Gomez</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Publicó hace 1 mes buscando reforzar el equipo de mercadeo de FP Moto, con la frase "las marcas más fuertes no se construyen únicamente con buenos productos, sino con experiencias memorables y con estrategia" — 1.469 seguidores, perfil público de LinkedIn</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Hola David. Vi tu publicación de hace un mes buscando reforzar el equipo de mercadeo de FP Moto — la frase sobre que las marcas fuertes no se construyen solo con buen producto, sino con experiencia y estrategia, se nota que la aplican en serio y no es una frase de relleno.
+Estoy construyendo Neggo, una plataforma en Medellín que conecta comercios con clientes verificados que ya están buscando su categoría — en este caso, motos. No reemplaza el trabajo de marca que ya vienen construyendo en FP, lo complementa: filtramos la parte de esa demanda que ya está lista para comprar, con score financiero antes de que llegue al equipo comercial. Cada comercio lo verificamos antes de listarlo, así el cliente sabe que quien lo contacta es real.
+A futuro estamos construyendo Neggo Ads, para que comercios aliados manejen también su pauta en Meta/Google desde la misma plataforma — si les interesa quedar en la lista de espera para cuando esté listo, les aviso.
+¿Tienen sentido 15 minutos esta semana para mostrarte cómo aplicaría puntualmente a FP Moto?</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>Armado</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>Categoría: Moto — primer perfil de esta categoría en el canal LinkedIn (tenía cero prospectos previos en el tracker). TRATAMIENTO DE CUENTA GRANDE aplicado (sección 6.1): marca establecida con equipo de mercadeo propio, contratación activa de un líder de ecosistema digital, 1.469 seguidores en el perfil del gerente — tono profesional, sin emoji, reconociendo su nivel antes de ofrecer, mención de Neggo Ads como lista de espera futura (evidencia: ads-ai-platform/ROADMAP.md). Mensaje listo — pendiente de envío por Jhey (no enviado).</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="331.2" customHeight="1">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Conector</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Esteban Cadavid</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Consultor Financiero para PYMES — marca personal "Hablemos de tu negocio", Medellín</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/estebancadavid/</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Carlos Guayara, Yady Alexandra Anzueta Duarte</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>Cuenta verificada, 2.993 seguidores, marca personal registrada como lugar de trabajo ("HABLEMOS DE TU NEGOCIO") y headline enfocado en flujo de caja predictivo para pymes, no en "vender más" — perfil público de LinkedIn</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>Hola Esteban. Vi tu perfil como consultor financiero para pymes — me llamó la atención que tu marca personal se llame justo "Hablemos de tu negocio", y que el foco esté en flujo de caja predictivo antes que en solo vender más.
+Estoy construyendo Neggo en Medellín: conectamos negocios locales con clientes ya verificados que buscan su servicio, con score financiero visible, y cobramos solo cuando el contacto es real, sin pauta de por medio. Buena parte de los pymes con los que hablas de flujo de caja seguramente también necesitan un canal de demanda que no dependa de pauta que no controlan.
+¿Vale la pena que lo conversemos, aunque sea para que me des tu mirada de consultor sobre si esto le sirve a la gente con la que trabajas?</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>Armado</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>Mensaje listo — pendiente de envío por Jhey (no enviado).</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="278.1" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Banco-Constructora</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Juan Pablo Rendón Pulgarín</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Coordinador Sala de Negocios — Constructora Capital, Medellín</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/juan-pablo-rend%C3%B3n-pulgar%C3%ADn-449684267/</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Mónica</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Rol específico como coordinador de la sala de negocios (ventas) de Constructora Capital en Medellín — perfil público de LinkedIn, sin Acerca de ni actividad reciente visible</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Hola Juan Pablo. Vi tu rol como coordinador de la sala de negocios en Constructora Capital, acá en Medellín.
+Estoy construyendo Neggo, una plataforma en etapa temprana que conecta clientes verificados con negocios y, a futuro, con constructoras por ciudad, estrato y presupuesto. Todavía no tengo nada formal para ofrecer del lado de constructoras — me interesa más entender cómo llega hoy el comprador a la sala de negocios, antes o después de la pauta, sin ninguna propuesta de por medio.
+¿Tienes 15 minutos esta semana para una charla informal, de fundador a alguien que está en el día a día de la sala de ventas?</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>Armado</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>EXPLORATORIO — sin pitch formal ni CTA de registro (regla secciones 9-10). Perfil pequeño (46 contactos), sin señales de cuenta grande — se mantiene el guion exploratorio estándar. Mensaje listo — pendiente de envío por Jhey (no enviado).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: gestionar respuestas reales y seguimientos de ventas
</commit_message>
<xml_diff>
--- a/docs/tracker-prospectos-neggo.xlsx
+++ b/docs/tracker-prospectos-neggo.xlsx
@@ -3235,7 +3235,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Esperar a que Jhey lo envíe</t>
+          <t>Revisar seguimiento sugerido y decidir si enviar</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -3245,7 +3245,7 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Cuenta grande (713 mil seguidores) — igual encaja en ICP Belleza/Spa Medellín, dirección confirmada en bio. Mensaje listo, pendiente de envío por Jhey (no enviado).</t>
+          <t>Cuenta grande (713 mil seguidores) — igual encaja en ICP Belleza/Spa Medellín, dirección confirmada en bio. Mensaje listo, pendiente de envío por Jhey (no enviado). | SEGUIMIENTO SUGERIDO (2026-08-06): Hola de nuevo — sé que el ritmo de Alma Prana es alto, así que quería retomar brevemente: seguimos viendo demanda real de spa para parejas en Medellín que hoy no se resuelve por un canal directo de leads calificados. Si tienen 5-10 minutos esta semana, les muestro cómo encajaría con las reservas de último minuto que ya vienen impulsando.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: agregar 3 perfiles nuevos a prospección Instagram (Celular, Carro, Moto)
</commit_message>
<xml_diff>
--- a/docs/tracker-prospectos-neggo.xlsx
+++ b/docs/tracker-prospectos-neggo.xlsx
@@ -3308,7 +3308,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="10.1640625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -4155,6 +4155,162 @@
         </is>
       </c>
     </row>
+    <row r="17" ht="126" customHeight="1">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>Comercio directo</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
+        <is>
+          <t>@next_technology__</t>
+        </is>
+      </c>
+      <c r="D17" s="10" t="inlineStr">
+        <is>
+          <t>Next Technology (NEXTECHNOLOGY) — Celular (venta de celulares y tecnología)</t>
+        </is>
+      </c>
+      <c r="E17" s="10" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/next_technology__/</t>
+        </is>
+      </c>
+      <c r="F17" s="10" t="inlineStr">
+        <is>
+          <t>Bio: "🖇️🖥️ E-commerce, Equipos con garantía y envío seguro, IMPORTADORES DIRECTOS" + "Tienda de telefonía celular". Dirección real: Calle 53 # 49-88N Opera Mall local F1-F3, Medellín, Antioquia. 39.832 seguidores, 637 publicaciones, cuenta muy activa (varios reels por semana), web nextechnology.com.co. Gancho real: reel de hace 4 días sobre el HONOR Play 10, cierra con "la confianza de comprar en una tienda física".</t>
+        </is>
+      </c>
+      <c r="G17" s="10" t="inlineStr">
+        <is>
+          <t>Hola equipo de Next Technology. Vi el reel del HONOR Play 10 de hace unos días — la parte donde mencionan "la confianza de comprar en una tienda física" me quedó sonando, porque es justo el problema que resolvemos del otro lado. Con casi 40 mil seguidores y punto físico en Opera Mall, ya tienen la marca resuelta. Estoy construyendo Neggo: llevamos personas de Medellín que ya buscan comprar un celular directo a comercios verificados — verificamos cada negocio antes de listarlo, así el cliente llega con confianza real, no solo con una promesa. No reemplaza lo que ya construyeron, filtra la demanda que ya está lista para comprar. También estamos armando Neggo Ads, para pautar en Meta/Google desde la misma plataforma — si les interesa la lista de espera para cuando esté listo, aviso. ¿Vemos 10 minutos cómo encaja?</t>
+        </is>
+      </c>
+      <c r="H17" s="10" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="I17" s="10" t="inlineStr">
+        <is>
+          <t>Armado</t>
+        </is>
+      </c>
+      <c r="J17" s="10" t="inlineStr">
+        <is>
+          <t>Categoría: Celular (antes en 0 prospectos). Cuenta grande/consolidada (39.832 seguidores, 637 publicaciones, actividad muy consistente) — tratamiento sección 6.1 aplicado (tono profesional, sin emoji de saludo, reconocimiento explícito antes del pitch, mención honesta de Neggo Ads en modo lista de espera). Mensaje listo, pendiente de envío por Jhey (no enviado).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="126" customHeight="1">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>Comercio directo</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t>@usadosdelnorte_</t>
+        </is>
+      </c>
+      <c r="D18" s="10" t="inlineStr">
+        <is>
+          <t>Usados del Norte — Carro (compra/venta/consignación de vehículos, SOAT, póliza todo riesgo)</t>
+        </is>
+      </c>
+      <c r="E18" s="10" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/usadosdelnorte_/</t>
+        </is>
+      </c>
+      <c r="F18" s="10" t="inlineStr">
+        <is>
+          <t>Bio: "🚗 Compra • Venta • Consignación de vehículos, 🤝 Vendemos tu carro al mejor precio, 💳 Crédito aprobado e..." Cuenta verificada, 19.812 seguidores, 1.783 publicaciones, web usadosdelnorte.netlify.app. Gancho real: post que advierte "Muchos carros en Medellín son robados, clonados o tienen problemas ocultos" y ofrece peritaje completo antes de comprar, cerrando con "te ayudamos a vender con confianza".</t>
+        </is>
+      </c>
+      <c r="G18" s="10" t="inlineStr">
+        <is>
+          <t>Hola equipo de Usados del Norte. Vi el post sobre carros robados o clonados en Medellín y el peritaje que hacen antes de la compra — es prácticamente el mismo problema que resolvemos nosotros, solo que del lado del cliente que busca el carro. Con casi 20 mil seguidores y cuenta verificada, ya tienen la confianza construida en el sector. Desde Neggo conectamos personas de Medellín que ya están buscando comprar un vehículo con comercios verificados como ustedes — cada comercio pasa una verificación antes de aparecer, y solo se paga cuando el lead es real, sin pauta fija. No compite con el trabajo de peritaje que ya hacen, lo complementa desde antes del primer contacto. ¿Hablamos 10 minutos esta semana?</t>
+        </is>
+      </c>
+      <c r="H18" s="10" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="I18" s="10" t="inlineStr">
+        <is>
+          <t>Armado</t>
+        </is>
+      </c>
+      <c r="J18" s="10" t="inlineStr">
+        <is>
+          <t>Categoría: Carro (antes en 0 prospectos). Cuenta grande/consolidada y verificada (19.812 seguidores, 1.783 publicaciones) — tratamiento sección 6.1 aplicado (tono profesional, sin emoji de saludo, reconocimiento explícito antes del pitch). Alineación temática fuerte: su propio pitch de peritaje ya habla de fraude/confianza, mismo terreno que el Sello de Confianza de Neggo. Mensaje listo, pendiente de envío por Jhey (no enviado).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="126" customHeight="1">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>Comercio directo</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>@compraventamedellin</t>
+        </is>
+      </c>
+      <c r="D19" s="10" t="inlineStr">
+        <is>
+          <t>Compraventa Medellín — Moto (compra/venta de motos usadas, recibe motos en parte de pago)</t>
+        </is>
+      </c>
+      <c r="E19" s="10" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/compraventamedellin/</t>
+        </is>
+      </c>
+      <c r="F19" s="10" t="inlineStr">
+        <is>
+          <t>Bio: "🛵200 Motos de segunda, Entrega Inmediata, 💥Recibimos tu moto en forma de pago, 💰Compramos tu moto, 📍Med..." Cuenta verificada, 381.263 seguidores, 38.188 publicaciones. Gancho real: post "¡TU PRÓXIMA MOTO ESTÁ AQUÍ!" con dirección real (Cra. 53 #38-34, Sector La Bayadera, Medellín) y motos desde $3.500.000.</t>
+        </is>
+      </c>
+      <c r="G19" s="10" t="inlineStr">
+        <is>
+          <t>Hola equipo de Compraventa Medellín. Con 381 mil seguidores y cuenta verificada, el alcance que ya tienen en Medellín no es fácil de igualar — se nota en el catálogo de motos listas para entrega inmediata que manejan en La Bayadera. Estoy construyendo Neggo: conectamos personas que ya están buscando comprar una moto con comercios verificados de la ciudad — revisamos cada comercio aliado antes de sumarlo a la plataforma, y el cliente llega con score financiero visible antes del primer contacto. No busca reemplazar el alcance que ya construyeron, sino entregarles la parte de esa demanda que ya está lista para comprar. También estamos armando Neggo Ads, para que comercios aliados gestionen pauta en Meta/Google desde la misma plataforma — si les interesa quedar en la lista de espera para cuando esté listo, aviso con gusto. ¿Vemos 10 minutos cómo encajaría con lo que ya tienen?</t>
+        </is>
+      </c>
+      <c r="H19" s="10" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="I19" s="10" t="inlineStr">
+        <is>
+          <t>Armado</t>
+        </is>
+      </c>
+      <c r="J19" s="10" t="inlineStr">
+        <is>
+          <t>Categoría: Moto (antes en 0 prospectos). Cuenta muy grande/consolidada y verificada (381.263 seguidores, 38.188 publicaciones) — tratamiento sección 6.1 aplicado (tono profesional, sin emoji de saludo, reconocimiento explícito antes del pitch, mención honesta de Neggo Ads en modo lista de espera). Mensaje listo, pendiente de envío por Jhey (no enviado).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId1"/>

</xml_diff>

<commit_message>
docs: agregar 3 perfiles nuevos a prospección LinkedIn (Carro, Conector, Banco-Constructora)
</commit_message>
<xml_diff>
--- a/docs/tracker-prospectos-neggo.xlsx
+++ b/docs/tracker-prospectos-neggo.xlsx
@@ -1592,7 +1592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K31"/>
+  <dimension ref="A1:K34"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -3293,6 +3293,172 @@
       <c r="K31" s="2" t="inlineStr">
         <is>
           <t>EXPLORATORIO — sin pitch formal ni CTA de registro (regla secciones 9-10, Fase 3 Bancos sigue bloqueada). Cuenta verificada, 1.317 seguidores — no aplica tratamiento de cuenta grande de la sección 6.1 (esa sección rige el pitch de comercios directos, no el segmento exploratorio). Mensaje listo — pendiente de envío por Jhey (no enviado).</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="126" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Comercio directo</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Julian E. Areiza C.</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>ALG Autos ⚪⚫ / Luxury Cars — concesionario especializado en vehículos de gama alta, Medellín</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/julian-e-areiza-c-82894a101/</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>La página de empresa de ALG Autos en LinkedIn se describe como especializada en "ofrecer una experiencia incomparable en la adquisición de vehículos de gama alta" — no un concesionario genérico. Perfil personal de Julian con 64 seguidores, sin Acerca de ni actividad reciente propia visible; el gancho real viene de la descripción pública de la empresa, no de la actividad personal.</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Hola, Julian. Vi que desde ALG Autos no manejan un concesionario genérico, sino que se especializan en vehículos de gama alta — se nota que el foco está puesto en la experiencia de compra, no solo en el inventario. Estoy construyendo Neggo, una plataforma que conecta negocios de Medellín con clientes que ya están buscando activamente ese tipo de vehículo, verificados y con score financiero antes de que te escriban. Cada negocio lo verificamos antes de listarlo, así el cliente sabe que el contacto es real. Pagás solo cuando el contacto es real, sin pauta ni permanencia, y los primeros 50 comercios de Medellín se quedan con el Sello de Confianza sin costo. ¿Tenés 10 minutos esta semana para que te cuente cómo aplicaría a ALG Autos?</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>Armado</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>Categoría: Carro — primer perfil de esta categoría en el canal LinkedIn (tenía cero prospectos previos en el tracker, junto con Celular y Computador, que se intentaron pero no arrojaron perfiles con suficiente base real de personalización esta corrida). Mensaje listo — pendiente de envío por Jhey (no enviado).</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="126" customHeight="1">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Conector</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>José I. (Iglesias B.)</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Cámara de Comercio de Medellín para Antioquia — Emprendedor, Consultor y Mentor | Estrategia, Gestión Comercial e Innovación, Medellín</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/joseiglesiasb/</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Marcela, Juan Sebastián y 6 contactos más (según LinkedIn)</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>Perfil verificado que trabaja en la Cámara de Comercio de Medellín para Antioquia. En su actividad reciente compartió y promovió un "Programa de Fortalecimiento Sectorial" dirigido al sector gastronómico, con acompañamiento técnico para mejorar productividad, tecnología e innovación en negocios reales — perfil público de LinkedIn.</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>Hola, José. Vi que trabajás en la Cámara de Comercio de Medellín para Antioquia, y entre tu actividad encontré el Programa de Fortalecimiento Sectorial que promoviste para el sector gastronómico — ese tipo de acompañamiento técnico a negocios reales es justo el terreno donde creo que Neggo puede sumar. Estoy construyendo Neggo: conectamos comercios de Medellín con clientes ya verificados que buscan su servicio, con score financiero visible, cobrando solo cuando el contacto es real. Muchos de los negocios que pasan por programas como el que impulsaste seguramente necesitan un canal de demanda que no dependa de pauta paga. ¿Te sirve que hablemos 10-15 minutos, aunque sea para que me digas si esto le hace sentido a la gente con la que trabajás?</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>Armado</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>Perfil verificado (ícono de verificación en LinkedIn). Mensaje listo — pendiente de envío por Jhey (no enviado).</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="126" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Banco-Constructora</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Carolina Zuleta</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Gerente Comercial — Desarrollo de Negocios, Estructuración y Gerencia de Proyectos, Constructora Convel S.A.S. (72+ años de trayectoria), Medellín</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/carolina-zuleta/</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Andrés (contacto en común, según LinkedIn)</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Publicó hace 5 días sobre el inicio de nuevos proyectos de Constructora Convel durante 2026, y en publicaciones recientes detalla proyectos reales en curso: Casa Nua Country (vivienda para adultos mayores), Wake Medellín (Design Hotels/Marriott International), Punta Vela Mall en Cartagena y DAVIarena — Convel destaca su trayectoria de más de 72 años como constructores. 2.865 seguidores, perfil público de LinkedIn, activo y publicando con frecuencia.</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>Hola, Carolina. Vi tu publicación de hace unos días sobre el inicio de nuevos proyectos de Constructora Convel este 2026 — con más de 72 años de trayectoria y proyectos tan distintos entre sí como Wake Medellín o Casa Nua Country, imagino que el perfil de comprador cambia bastante de un proyecto a otro. Estoy construyendo Neggo, una plataforma en etapa temprana que conecta clientes verificados con negocios en Medellín y, a futuro, con constructoras por ciudad, estrato y presupuesto. Todavía no tengo nada formal para ofrecer del lado de constructoras — me interesa más entender cómo filtran hoy quién realmente tiene el perfil financiero para cada proyecto antes de invertir tiempo comercial en esa persona, sin ninguna propuesta de por medio. ¿Tenés 15 minutos en las próximas semanas para una charla informal sobre cómo lo resuelven hoy en Convel?</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>Armado</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>EXPLORATORIO — sin pitch formal ni CTA de registro (regla secciones 9-10). Cuenta activa con 2.865 seguidores y trayectoria real de la constructora (72+ años) — no aplica tratamiento de cuenta grande de la sección 6.1 (esa sección rige el pitch de comercios directos, no el segmento exploratorio de Banco-Constructora, mismo criterio ya usado con Jorge Montoya Tobón y Juan Pablo Arce Fernández). Mensaje listo — pendiente de envío por Jhey (no enviado).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: agregar 4 perfiles nuevos a prospección Instagram (Viaje, Carro, Educación, Moto)
</commit_message>
<xml_diff>
--- a/docs/tracker-prospectos-neggo.xlsx
+++ b/docs/tracker-prospectos-neggo.xlsx
@@ -4148,7 +4148,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J27"/>
+  <dimension ref="A1:J31"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="10.1640625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -5567,6 +5567,214 @@
         </is>
       </c>
     </row>
+    <row r="28" ht="126" customHeight="1">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B28" s="10" t="inlineStr">
+        <is>
+          <t>Comercio directo</t>
+        </is>
+      </c>
+      <c r="C28" s="10" t="inlineStr">
+        <is>
+          <t>@malemotours</t>
+        </is>
+      </c>
+      <c r="D28" s="10" t="inlineStr">
+        <is>
+          <t>Malemo Tours — Viaje (agencia de viajes: tours, hoteles, vuelos, cruceros)</t>
+        </is>
+      </c>
+      <c r="E28" s="10" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/malemotours/</t>
+        </is>
+      </c>
+      <c r="F28" s="10" t="inlineStr">
+        <is>
+          <t>Bio: "Agencia de viajes ✈️🌍 Tu puerta a aventuras inolvidables: tours, hoteles, vuelos, y cruceros. ¡Viaja con nosotros!". 1.646 seguidores, 61 publicaciones. Gancho real: post de hace 2 semanas anunciando su primer tour en colaboración con @bizcochitoshow y @ruddy.vicioso, itinerario por "Medellín, la Ciudad de la Eterna Primavera".</t>
+        </is>
+      </c>
+      <c r="G28" s="10" t="inlineStr">
+        <is>
+          <t>Hola Malemo Tours 👋 Vi el post del primer tour en conjunto con @bizcochitoshow y @ruddy.vicioso por Medellín, "la ciudad de la eterna primavera" — buena forma de sumar público nuevo. Desde Neggo conectamos personas que ya buscan agencia de viajes en Medellín con negocios como el suyo, y solo se paga cuando el lead es real, sin pauta fija ni permanencia. ¿Le cuento en 5 minutos cómo funciona?</t>
+        </is>
+      </c>
+      <c r="H28" s="10" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="I28" s="10" t="inlineStr">
+        <is>
+          <t>Armado</t>
+        </is>
+      </c>
+      <c r="J28" s="10" t="inlineStr">
+        <is>
+          <t>Categoría: Viaje (antes en 1 prospecto). Cuenta pequeña pero real y activa (1.646 seguidores, 61 publicaciones) — tono estándar sección 4. Mensaje listo, pendiente de envío por Jhey (no enviado).</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="126" customHeight="1">
+      <c r="A29" s="10" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B29" s="10" t="inlineStr">
+        <is>
+          <t>Comercio directo</t>
+        </is>
+      </c>
+      <c r="C29" s="10" t="inlineStr">
+        <is>
+          <t>@apjcentroautomotriz</t>
+        </is>
+      </c>
+      <c r="D29" s="10" t="inlineStr">
+        <is>
+          <t>APJ Centro Automotriz — Carro (taller de reparación de automóviles)</t>
+        </is>
+      </c>
+      <c r="E29" s="10" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/apjcentroautomotriz/</t>
+        </is>
+      </c>
+      <c r="F29" s="10" t="inlineStr">
+        <is>
+          <t>Bio: "Taller de reparación de automóviles 📍Calle 73 # 72C - 95 Robledo Pilarica. Diagnóstico y mantenimiento profesional. Atención a flotas, particulares...". 568 seguidores, 99 publicaciones, WhatsApp real en bio. Gancho real: grid de publicaciones recientes cubre cambio de aceite, latonería/pintura, mantenimiento de ejes/suspensión, frenos y batería/alternador — no solo un servicio único.</t>
+        </is>
+      </c>
+      <c r="G29" s="10" t="inlineStr">
+        <is>
+          <t>Hola equipo de APJ 👋 Vi que además del cambio de aceite también cubren frenos, batería y suspensión — no es un taller de una sola cosa. En Neggo llevamos personas de Medellín que ya buscan un taller de confianza a comercios como el suyo, verificamos cada negocio antes de listarlo y solo cobramos si el lead es real, sin pauta fija. ¿Vemos 5 minutos cómo encaja con lo que hacen en Robledo Pilarica?</t>
+        </is>
+      </c>
+      <c r="H29" s="10" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="I29" s="10" t="inlineStr">
+        <is>
+          <t>Armado</t>
+        </is>
+      </c>
+      <c r="J29" s="10" t="inlineStr">
+        <is>
+          <t>Categoría: Carro (antes en 1 prospecto). Cuenta pequeña pero real y activa (568 seguidores, 99 publicaciones, dirección y WhatsApp reales) — tono estándar sección 4, mención concreta de verificación (Sello de Confianza) sin usarlo como etiqueta vacía. Mensaje listo, pendiente de envío por Jhey (no enviado).</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="126" customHeight="1">
+      <c r="A30" s="10" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B30" s="10" t="inlineStr">
+        <is>
+          <t>Comercio directo</t>
+        </is>
+      </c>
+      <c r="C30" s="10" t="inlineStr">
+        <is>
+          <t>@upainscripciones</t>
+        </is>
+      </c>
+      <c r="D30" s="10" t="inlineStr">
+        <is>
+          <t>Instituto Técnico Unidos por Antioquia — Educación (formación técnica en salud y estética, Bello)</t>
+        </is>
+      </c>
+      <c r="E30" s="10" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/upainscripciones/</t>
+        </is>
+      </c>
+      <c r="F30" s="10" t="inlineStr">
+        <is>
+          <t>Bio: "instituto tecnico unidos por Antioquia. Desde 1987 formamos a comunidades en salud y cuidado, mejorando vidas con educación, empatía y vocación." Dirección real: Av 50a #53-07, Bello, Antioquia. 611 seguidores, 163 publicaciones, WhatsApp real en bio. Gancho real: post de hace 1 semana sobre programa de Micropigmentación de Cejas y Labios 100% presencial, cupos limitados, matrículas abiertas, tel 304 415 7632.</t>
+        </is>
+      </c>
+      <c r="G30" s="10" t="inlineStr">
+        <is>
+          <t>Hola equipo del Instituto Unidos por Antioquia. Llevan desde 1987 formando gente en salud y cuidado — no es una academia que recién arranca, es trayectoria real de casi 40 años. Estoy construyendo Neggo: conectamos personas de Medellín que ya buscan un curso o certificación (como el de Micropigmentación que abrieron esta semana) con instituciones serias como la suya, con score financiero verificado antes de que el contacto llegue al chat. No reemplaza la formación que ya ofrecen, filtra la demanda que ya está lista para matricularse. Cumplimos la Ley 1581 de protección de datos con la información de cada estudiante. ¿Hablamos 10 minutos esta semana?</t>
+        </is>
+      </c>
+      <c r="H30" s="10" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="I30" s="10" t="inlineStr">
+        <is>
+          <t>Armado</t>
+        </is>
+      </c>
+      <c r="J30" s="10" t="inlineStr">
+        <is>
+          <t>Categoría: Educación (antes en 1 prospecto). Trayectoria reconocible (39 años operando, instituto técnico formal) aplica criterio de cuenta grande/consolidada aunque los seguidores sean bajos (611) — tratamiento sección 6.1 aplicado (tono profesional, sin emoji de saludo, reconocimiento explícito antes del pitch). Ubicado en Bello (área metropolitana de Medellín/Valle de Aburrá, mismo criterio ya usado con Itagüí en fila 19). Mensaje listo, pendiente de envío por Jhey (no enviado).</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="126" customHeight="1">
+      <c r="A31" s="10" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B31" s="10" t="inlineStr">
+        <is>
+          <t>Comercio directo</t>
+        </is>
+      </c>
+      <c r="C31" s="10" t="inlineStr">
+        <is>
+          <t>@motosracingmed</t>
+        </is>
+      </c>
+      <c r="D31" s="10" t="inlineStr">
+        <is>
+          <t>Motos Racing Medellín — Moto (servicio técnico especializado KTM, Husqvarna, Dominar, Envigado)</t>
+        </is>
+      </c>
+      <c r="E31" s="10" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/motosracingmed/</t>
+        </is>
+      </c>
+      <c r="F31" s="10" t="inlineStr">
+        <is>
+          <t>Bio: "Servicio técnico especializado para motos 🏍️ Expertos en KTM y Dominar. Diagnóstico, mantenimiento y reparación...". Ubicación real: Envigado. 1.165 seguidores, 210 publicaciones, WhatsApp real en bio. Gancho real: post de hace 7 semanas explicando por qué una KTM, Husqvarna o Dominar "no llegan a cualquier taller" y detallando su proceso (diagnóstico, procedimientos con criterio técnico, seguridad primero).</t>
+        </is>
+      </c>
+      <c r="G31" s="10" t="inlineStr">
+        <is>
+          <t>Hola equipo de Motos Racing 👋 Vi el post sobre por qué una KTM o Husqvarna no debería llegar a cualquier taller — se nota que no es solo cambiar aceite. Desde Neggo conectamos motociclistas de Medellín que ya buscan taller especializado con negocios como el suyo en Envigado, y solo pagan cuando el lead es real, sin pauta fija ni permanencia. ¿Le cuento en 5 minutos cómo funciona?</t>
+        </is>
+      </c>
+      <c r="H31" s="10" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="I31" s="10" t="inlineStr">
+        <is>
+          <t>Armado</t>
+        </is>
+      </c>
+      <c r="J31" s="10" t="inlineStr">
+        <is>
+          <t>Categoría: Moto (antes en 1 prospecto). Cuenta pequeña pero real y activa (1.165 seguidores, 210 publicaciones, ubicación Envigado confirmada, WhatsApp real) — tono estándar sección 4. Mensaje listo, pendiente de envío por Jhey (no enviado).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId1"/>

</xml_diff>

<commit_message>
tracker: agregar 15 propuestas personalizadas para talleres carro/moto (fotos de negocios)
</commit_message>
<xml_diff>
--- a/docs/tracker-prospectos-neggo.xlsx
+++ b/docs/tracker-prospectos-neggo.xlsx
@@ -507,7 +507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K20"/>
+  <dimension ref="A1:K35"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1577,6 +1577,828 @@
       <c r="K20" s="2" t="inlineStr">
         <is>
           <t>Mensaje listo — pendiente de envío por Jhey (no enviado)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>El Amigo De Las Motos</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Moto</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Facebook @elamigodelasmotos.co / WhatsApp 316 5446054</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Medellín</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Expertos en electricidad de motos (ramales, bobinado), reel con ~798K vistas, 15K seguidores FB</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Hola! Te escribo porque estamos construyendo Neggo, y queremos que un taller como el tuyo haga parte.
+Vi tu contenido sobre electricidad de motos — el reel del Yamaha DT que llegó desde Caquetá tiene casi 100 mil vistas, se nota que la gente confía en lo que mostrás y en cómo explicás el trabajo.
+Hemos visto que muchas personas dejan de llevar la moto a un taller nuevo por miedo: van con un problema puntual y terminan con más daños, o nadie les da garantía real. Eso hace que un buen taller como el tuyo tenga que competir contra la desconfianza de otros, no contra su propio trabajo.
+En Neggo verificamos cada taller antes de que aparezca — el cliente llega ya con confianza, no adivinando. ¿Tenés 10 minutos esta semana para contarte cómo funciona?</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Armado</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo revise y envíe</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Cuenta con buen alcance (15K+, reels virales) — tono cercano pero ya reconociendo su nivel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>AutoReel Medellín</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Carro</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Facebook (Publicidad) / WhatsApp 311 372 0142</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>El Poblado, Medellín</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Afinación profesional de motor diésel (limpieza inyección, turbo, EGR)</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Hola! Estamos construyendo Neggo y queremos que un taller como AutoReel haga parte.
+Vi que se especializan en afinación de motor diésel — limpieza de inyección, turbo, EGR, ese nivel de detalle no lo hace cualquier taller en Medellín.
+Hemos visto que mucha gente evita llevar su carro a un taller nuevo por una mala experiencia: entran con un problema y salen con tres, sin ninguna garantía. Eso golpea también a los talleres que sí hacen las cosas bien, porque el cliente ya no confía a ciegas.
+En Neggo verificamos cada taller antes de listarlo, así el cliente llega con la confianza ya puesta. ¿Tenés 10 minutos esta semana para que te cuente cómo funciona?</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Armado</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo revise y envíe</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Especializado diésel — ticket alto potencial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Vehifrenos Medellín</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Carro</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Facebook (Publicidad) / WhatsApp 318 7006090</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Medellín</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Contenido de prevención (disco a punto de rayarse), enfoque en revisión preventiva</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Hola! Te escribo porque estamos construyendo Neggo y queremos que un taller como Vehifrenos haga parte.
+Vi el video donde muestran el disco a punto de rayarse antes de que sea tarde — ese enfoque en prevención es justo lo que mucha gente no encuentra en un taller.
+Es común que alguien posponga una revisión de frenos por miedo a caer con un taller que le dañe más de lo que tenía, o que no le explique nada. Eso frena ventas que ustedes sí se merecen.
+En Neggo verificamos cada taller antes de aparecer — el cliente llega ya con confianza. ¿Tenés 10 minutos esta semana para contarte cómo funciona?</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Armado</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo revise y envíe</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Especialista en frenos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Autollantas Nutibara</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Carro</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Facebook (Publicidad) / WhatsApp 322 5040552</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Medellín</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>50 años de experiencia, alineación/balanceo, frenos, batería, llantas Goodyear/Michelin/BFGoodrich</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Buenas tardes. Los 50 años de Autollantas Nutibara ya son una carta de presentación que pocos talleres en Medellín pueden mostrar — no es algo que se pueda inventar.
+Le escribo porque estamos construyendo Neggo, pensado como un complemento a lo que un taller con su trayectoria ya construyó: hoy mucha gente evita probar un taller nuevo por miedo a una mala experiencia (entrar con un problema y salir con tres, sin garantía real). Nosotros verificamos cada taller antes de aparecer en la plataforma, así el cliente llega a ustedes ya con la confianza puesta, no comparando a ciegas contra talleres sin trayectoria.
+¿Tendría 10-15 minutos esta semana para contarle cómo funciona y qué sentido tendría para un taller de su nivel?</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Armado</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo revise y envíe</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>CUENTA GRANDE (50 años, marca establecida) — tono profesional aplicado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>ServiVag</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Carro</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Facebook (Publicidad) / WhatsApp 313 7447537</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Medellín</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Especialistas Audi/Volkswagen, técnicos certificados en marcas premium, 20% dcto primer mantenimiento</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Hola! Estamos construyendo Neggo y queremos que un taller como ServiVag haga parte.
+Vi que se especializan en Audi y Volkswagen con técnicos certificados en marcas premium — ese nivel de especialización es exactamente lo que un dueño de un carro de alta gama busca y no siempre encuentra.
+Muchas personas con vehículos así evitan un taller nuevo por miedo a que no sepan tratar su carro, o que salgan con más daños de los que llegaron. En Neggo verificamos cada taller antes de listarlo — el cliente llega ya con confianza, no adivinando.
+¿Tenés 10 minutos esta semana para contarte cómo funciona?</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Armado</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo revise y envíe</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>TICKET ALTO — vehículos premium, candidato a CPL superior (señalar en la llamada, no en el mensaje).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Serviteca Md (Dixtrifiltros)</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Carro</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Facebook (Publicidad) / WhatsApp 310 3806429</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Medellín</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Cambio de aceite desde $98.000, mantenimiento preventivo, lubricación y filtración</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Hola! Te escribo porque estamos construyendo Neggo y queremos que un taller como el suyo haga parte.
+Vi que tienen cambio de aceite desde $98.000 con un enfoque real en mantenimiento preventivo — ese tipo de claridad en precio es algo que a muchos clientes les da tranquilidad desde el primer contacto.
+Hemos visto que mucha gente pospone hasta el mantenimiento básico por desconfianza de talleres que suman cosas no pedidas o no explican bien qué están cobrando. En Neggo verificamos cada taller antes de aparecer, así el cliente llega ya confiando en lo que le van a decir.
+¿Tenés 10 minutos esta semana para contarte cómo funciona?</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Armado</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo revise y envíe</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Servicio de entrada (cambio de aceite) — buen gancho de precio claro.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Serviteck Automotriz</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Carro</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Facebook (Publicidad) / WhatsApp 333 2823505</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Medellín</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Buen engagement real (183 likes, 18 comentarios) en su contenido</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Hola! Estamos construyendo Neggo y queremos que un taller como Serviteck Automotriz haga parte.
+Vi la interacción real que generan sus publicaciones — se nota que ya tienen una comunidad que confía en lo que muestran.
+Es común que alguien dude antes de llevar su carro a un taller que no conoce, por miedo a salir con más problemas de los que llegó. En Neggo resolvemos justo eso: verificamos cada taller antes de que aparezca, para que el cliente llegue con la confianza ya puesta.
+¿Tenés 10 minutos esta semana para contarte cómo funciona?</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Armado</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo revise y envíe</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Ingenio Mecánico</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Carro</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Instagram @ingeniomecanicomed / WhatsApp 573245121897</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Laureles, Medellín</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Ya se posicionan como 'Centro de Servicios Automotriz de Confianza', cuenta verificada, secciones de Casos de Éxito y Testimonios, especialistas Mazda</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Hola! Te escribo porque estamos construyendo Neggo y su taller me llamó la atención apenas vi el perfil.
+Ya hablan de ser 'tu Centro de Servicios Automotriz de Confianza' — literalmente lo dice su bio — y tienen hasta una sección de Casos de Éxito y Testimonios. Eso es exactamente lo que Neggo busca resaltar de los talleres que sí trabajan bien.
+El problema es que la mayoría de los clientes no puede distinguir entre un taller como el de ustedes y uno que promete lo mismo pero no cumple — muchos entran con un problema y salen con tres, sin garantía. Nosotros verificamos cada taller antes de listarlo, así el cliente llega a ustedes ya sabiendo que es real.
+¿Tenés 10 minutos esta semana para contarte cómo funciona?</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Armado</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo revise y envíe</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>Verificado, 1.7K seguidores, ya usa lenguaje de confianza como su propia bandera — encaje muy fuerte con el mensaje de Neggo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Autolex</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Carro</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Instagram @autolex_serviteca_ / WhatsApp 313 569 1835</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Envigado</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Más de 10 años, ya hace parte de una red 'Talleres Aliados / Importadoras Asociadas', revisión general gratis con cambio de aceite</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Buenas! Le escribo porque estamos construyendo Neggo y AUTOLEX me pareció un caso interesante — ya hacen parte de una red de Talleres Aliados con Importadoras Asociadas, y tienen más de 10 años cuidando motores en Envigado.
+Eso demuestra algo que Neggo también busca resolver del otro lado: mucha gente no sabe distinguir un taller confiable de uno que no lo es, y termina evitando probar talleres nuevos por miedo a salir con más daños de los que llegó. Nosotros verificamos cada taller antes de listarlo en la plataforma, para que el cliente llegue ya con la confianza puesta — algo que complementa la red que ya construyeron, no la reemplaza.
+¿Tendrían 10-15 minutos esta semana para conversar?</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Armado</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo revise y envíe</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>CUENTA GRANDE (red de talleres aliados, +10 años) — tono profesional aplicado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Shopping CARSS MED</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Carro</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Facebook (Publicidad) / WhatsApp 322 5192109</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Medellín</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Latonería/pintura de alto nivel (Land Cruiser Prado 2012 actualizada a 2024, body kit, tapizado)</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Hola! Estamos construyendo Neggo y queremos que un taller como Shopping CARSS haga parte.
+Vi el trabajo que hicieron en la Land Cruiser Prado 2012 actualizada a 2024 — pintura, body kit, tapizado — ese nivel de detalle no lo tiene cualquier taller.
+Mucha gente con un carro de ese valor evita un taller nuevo por miedo a que no lo traten con el cuidado que merece. En Neggo verificamos cada taller antes de listarlo, así el cliente llega ya con la confianza puesta, sin arriesgarse a adivinar.
+¿Tenés 10 minutos esta semana para contarte cómo funciona?</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Armado</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo revise y envíe</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>TICKET ALTO — latonería/pintura de vehículos de alto valor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Cars System CSS</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Carro</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Facebook (Publicidad, verificado) / WhatsApp 311 4009045</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Medellín</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Servicio de PDR (extracción de golpes sin pintar), cuenta verificada</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Hola! Te escribo porque estamos construyendo Neggo y queremos que un taller como Cars System haga parte.
+Vi el servicio de PDR (extracción de golpes sin pintar) — es un servicio que mucha gente ni sabe que existe, y cuando lo necesita no sabe en quién confiar para hacerlo bien.
+Hemos visto que la gente pospone estas reparaciones por miedo a caer con alguien que dañe más el carro. En Neggo verificamos cada taller antes de aparecer, así el cliente llega ya confiando en el trabajo que va a recibir.
+¿Tenés 10 minutos esta semana para contarte cómo funciona?</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Armado</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo revise y envíe</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Todorines</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Carro</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Facebook / WhatsApp 314 6385481</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Medellín (+ Bello, Sabaneta, Envigado, Itagüí)</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>15 años de experiencia en rines y llantas, presencia multi-sede en el Área Metropolitana, web propia</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Buenas! Le escribo porque estamos construyendo Neggo y Todorines me pareció un caso interesante — 15 años de experiencia y presencia en Medellín, Bello, Sabaneta, Envigado e Itagüí no es algo que cualquiera pueda mostrar.
+Le cuento por qué le escribo: mucha gente evita comprar rines o llantas en un lugar que no conoce por miedo a que le vendan algo de mala calidad o mal instalado. Eso frena ventas incluso para negocios como el suyo, con trayectoria real. En Neggo verificamos cada negocio antes de listarlo, así el cliente llega ya con la confianza puesta, sin comparar a ciegas.
+¿Tendría 10-15 minutos esta semana para contarle cómo funciona?</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Armado</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo revise y envíe</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>CUENTA GRANDE (15 años, multi-sede, web propia) — tono profesional aplicado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Baterías para carro Medellín</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Carro</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Facebook (Publicidad) / WhatsApp 333 7313605</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Medellín y Valle de Aburrá</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Diagnóstico gratis antes de vender, servicio a domicilio 24/7, marcas Varta/Mac/Tudor/Duncan/Willard</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Hola! Estamos construyendo Neggo y queremos que un negocio como Baterías para Carro Medellín haga parte.
+Vi que ofrecen diagnóstico gratis antes de vender nada — eso ya dice mucho, porque hemos visto que la gente desconfía justo de eso: que le vendan una batería nueva cuando el problema real era otro.
+En Neggo verificamos cada negocio antes de que aparezca, así el cliente llega confiando en que le van a decir la verdad, no solo a venderle. ¿Tenés 10 minutos esta semana para contarte cómo funciona?</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Armado</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo revise y envíe</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Baterías a domicilio 24 Horas</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Carro</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Facebook (Publicidad) / WhatsApp 320 6692767</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Medellín-Antioquia</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Domicilio e instalación gratis 24/7, bono de descuento $60.000</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Hola! Te escribo porque estamos construyendo Neggo y queremos que un negocio como el suyo haga parte.
+Vi que manejan domicilio e instalación gratis 24/7 en Medellín — para alguien varado con el carro sin batería, esa rapidez es justo lo que necesita, pero también lo que más aprovechan los que no son serios.
+Hemos visto que mucha gente duda antes de llamar a un desconocido a esa hora, por miedo a que le cobren de más o le instalen algo de mala calidad. En Neggo verificamos cada negocio antes de listarlo, así el cliente llega ya confiando en que es real. ¿Tenés 10 minutos esta semana para contarte cómo funciona?</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Armado</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo revise y envíe</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Competidor directo de Baterías para carro Medellín — mensaje con gancho distinto (velocidad/domicilio vs. diagnóstico honesto).</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Autosafecol</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Carro</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Facebook / WhatsApp 311 8274967</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Perpetuo Socorro, Medellín</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Electrónica automotriz</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Hola! Estamos construyendo Neggo y queremos que un negocio como Autosafecol haga parte.
+La electrónica de un carro es de lo que más desconfianza genera — mucha gente no sabe si el problema real era lo que le dijeron, o si terminó pagando por algo que no necesitaba.
+En Neggo verificamos cada negocio antes de que aparezca, así el cliente llega ya con la confianza puesta, no adivinando. ¿Tenés 10 minutos esta semana para contarte cómo funciona?</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Armado</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo revise y envíe</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Categoría Electrónica — verificar subcategoría exacta en la llamada.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
tracker: Baterías a Domicilio 24 Horas respondió, seguimiento armado
</commit_message>
<xml_diff>
--- a/docs/tracker-prospectos-neggo.xlsx
+++ b/docs/tracker-prospectos-neggo.xlsx
@@ -1624,7 +1624,6 @@
           <t>Armado</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr">
         <is>
           <t>Esperar a que Jhey lo revise y envíe</t>
@@ -1680,7 +1679,6 @@
           <t>Armado</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr">
         <is>
           <t>Esperar a que Jhey lo revise y envíe</t>
@@ -1736,7 +1734,6 @@
           <t>Armado</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr">
         <is>
           <t>Esperar a que Jhey lo revise y envíe</t>
@@ -1791,7 +1788,6 @@
           <t>Armado</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr">
         <is>
           <t>Esperar a que Jhey lo revise y envíe</t>
@@ -1847,7 +1843,6 @@
           <t>Armado</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr">
         <is>
           <t>Esperar a que Jhey lo revise y envíe</t>
@@ -1903,7 +1898,6 @@
           <t>Armado</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr">
         <is>
           <t>Esperar a que Jhey lo revise y envíe</t>
@@ -1959,13 +1953,11 @@
           <t>Armado</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr">
         <is>
           <t>Esperar a que Jhey lo revise y envíe</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2011,7 +2003,6 @@
           <t>Armado</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr">
         <is>
           <t>Esperar a que Jhey lo revise y envíe</t>
@@ -2066,7 +2057,6 @@
           <t>Armado</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr">
         <is>
           <t>Esperar a que Jhey lo revise y envíe</t>
@@ -2122,7 +2112,6 @@
           <t>Armado</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr">
         <is>
           <t>Esperar a que Jhey lo revise y envíe</t>
@@ -2178,13 +2167,11 @@
           <t>Armado</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr">
         <is>
           <t>Esperar a que Jhey lo revise y envíe</t>
         </is>
       </c>
-      <c r="K31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2229,7 +2216,6 @@
           <t>Armado</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr">
         <is>
           <t>Esperar a que Jhey lo revise y envíe</t>
@@ -2284,13 +2270,11 @@
           <t>Armado</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr">
         <is>
           <t>Esperar a que Jhey lo revise y envíe</t>
         </is>
       </c>
-      <c r="K33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2332,18 +2316,26 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Armado</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr"/>
+          <t>Respondió</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Hola Daniel! Con gusto te cuento.
+Neggo es una plataforma donde la gente busca negocios de confianza para resolver algo puntual — en tu caso, alguien que necesita cambiar la batería del carro, muchas veces varado o con afán. Nosotros verificamos cada negocio antes de que aparezca en la plataforma, así el cliente que te contacta ya llega confiando en que sos real y serio, no adivinando entre opciones.
+Lo que buscamos con vos es que Baterías a Domicilio 24 Horas esté ahí como una opción verificada — con tu servicio de domicilio e instalación gratis 24/7, que ya es un diferencial fuerte frente a otros.
+El modelo de pago es flexible, lo vemos según lo que te sirva más a vos: podés pagar por cada cliente que te enviamos, o solo cuando ese cliente efectivamente te compra. Nada fijo todavía, lo conversamos según cómo trabajás.
+¿Tenés 10-15 minutos esta semana, una llamada rápida o seguimos por acá, para contarte los detalles completos?</t>
+        </is>
+      </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Esperar a que Jhey lo revise y envíe</t>
+          <t>Esperar respuesta de Daniel / agendar llamada si acepta</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>Competidor directo de Baterías para carro Medellín — mensaje con gancho distinto (velocidad/domicilio vs. diagnóstico honesto).</t>
+          <t>Competidor directo de Baterías para carro Medellín — mensaje con gancho distinto (velocidad/domicilio vs. diagnóstico honesto). | RESPONDIÓ (10 ago) — Daniel Marín pidió más info, se le explicó el mecanismo y modelo de pago abierto.</t>
         </is>
       </c>
     </row>
@@ -2390,7 +2382,6 @@
           <t>Armado</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr">
         <is>
           <t>Esperar a que Jhey lo revise y envíe</t>

</xml_diff>

<commit_message>
tracker: Autolex respondió, seguimiento armado (tono cuenta grande)
</commit_message>
<xml_diff>
--- a/docs/tracker-prospectos-neggo.xlsx
+++ b/docs/tracker-prospectos-neggo.xlsx
@@ -78,6 +78,7 @@
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -113,7 +114,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -140,6 +141,10 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -510,19 +515,19 @@
   <dimension ref="A1:K35"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="60" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="45" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" style="11" min="1" max="1"/>
+    <col width="24" customWidth="1" style="11" min="2" max="2"/>
+    <col width="22.6640625" customWidth="1" style="11" min="3" max="3"/>
+    <col width="49.6640625" bestFit="1" customWidth="1" style="11" min="4" max="4"/>
+    <col width="24" customWidth="1" style="11" min="5" max="5"/>
+    <col width="82.83203125" customWidth="1" style="11" min="6" max="6"/>
+    <col width="60" customWidth="1" style="11" min="7" max="7"/>
+    <col width="18" customWidth="1" style="11" min="8" max="8"/>
+    <col width="13" customWidth="1" style="11" min="9" max="9"/>
+    <col width="45" customWidth="1" style="11" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1" ht="56" customHeight="1">
+    <row r="1" ht="56" customHeight="1" s="11">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Fecha</t>
@@ -579,7 +584,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="98" customHeight="1">
+    <row r="2" ht="98" customHeight="1" s="11">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
@@ -631,7 +636,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="84" customHeight="1">
+    <row r="3" ht="84" customHeight="1" s="11">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
@@ -683,7 +688,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="84" customHeight="1">
+    <row r="4" ht="84" customHeight="1" s="11">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
@@ -735,7 +740,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="84" customHeight="1">
+    <row r="5" ht="84" customHeight="1" s="11">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
@@ -787,7 +792,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="370" customHeight="1">
+    <row r="6" ht="370" customHeight="1" s="11">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
@@ -847,7 +852,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="98" customHeight="1">
+    <row r="7" ht="98" customHeight="1" s="11">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
@@ -899,7 +904,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="140" customHeight="1">
+    <row r="8" ht="140" customHeight="1" s="11">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
@@ -958,7 +963,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="84" customHeight="1">
+    <row r="9" ht="84" customHeight="1" s="11">
       <c r="A9" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
@@ -1010,7 +1015,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="224" customHeight="1">
+    <row r="10" ht="224" customHeight="1" s="11">
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
@@ -1067,7 +1072,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="98" customHeight="1">
+    <row r="11" ht="98" customHeight="1" s="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
@@ -1115,7 +1120,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="84" customHeight="1">
+    <row r="12" ht="84" customHeight="1" s="11">
       <c r="A12" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
@@ -1167,7 +1172,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="84" customHeight="1">
+    <row r="13" ht="84" customHeight="1" s="11">
       <c r="A13" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
@@ -1215,7 +1220,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="84" customHeight="1">
+    <row r="14" ht="84" customHeight="1" s="11">
       <c r="A14" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
@@ -1263,7 +1268,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="84" customHeight="1">
+    <row r="15" ht="84" customHeight="1" s="11">
       <c r="A15" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
@@ -1315,7 +1320,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="192" customHeight="1">
+    <row r="16" ht="192" customHeight="1" s="11">
       <c r="A16" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
@@ -1351,7 +1356,7 @@
           <t>Hola 👋 Vi sus spa days y planes de pareja en Laureles. Te escribo porque en Neggo conectamos negocios de Medellín con clientes que ya están buscando activamente su servicio — no es publicidad genérica, es gente que pidió contacto directo. Pagas solo por resultado real (CPL bajo), sin pauta ni permanencia. ¿Te interesa que te cuente en 5 min cómo funciona?</t>
         </is>
       </c>
-      <c r="H16" s="8" t="inlineStr">
+      <c r="H16" s="12" t="inlineStr">
         <is>
           <t>Hola, bienvenido a Amatsu spa, puedes comunicarte con nosotros a traves del whatsApp 3186506537 para hacer tus consultas y reserva.o si desea le responderemos por aca, mas tarde, Gracias por preferirnos.</t>
         </is>
@@ -1372,7 +1377,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="84" customHeight="1">
+    <row r="17" ht="84" customHeight="1" s="11">
       <c r="A17" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
@@ -1424,7 +1429,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="84" customHeight="1">
+    <row r="18" ht="84" customHeight="1" s="11">
       <c r="A18" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
@@ -1476,7 +1481,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="84" customHeight="1">
+    <row r="19" ht="84" customHeight="1" s="11">
       <c r="A19" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
@@ -1528,7 +1533,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="84" customHeight="1">
+    <row r="20" ht="84" customHeight="1" s="11">
       <c r="A20" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
@@ -1580,7 +1585,7 @@
         </is>
       </c>
     </row>
-    <row r="21">
+    <row r="21" ht="240" customHeight="1" s="11">
       <c r="A21" t="inlineStr">
         <is>
           <t>2026-08-10</t>
@@ -1611,7 +1616,7 @@
           <t>Expertos en electricidad de motos (ramales, bobinado), reel con ~798K vistas, 15K seguidores FB</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="G21" s="12" t="inlineStr">
         <is>
           <t>Hola! Te escribo porque estamos construyendo Neggo, y queremos que un taller como el tuyo haga parte.
 Vi tu contenido sobre electricidad de motos — el reel del Yamaha DT que llegó desde Caquetá tiene casi 100 mil vistas, se nota que la gente confía en lo que mostrás y en cómo explicás el trabajo.
@@ -1621,7 +1626,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Armado</t>
+          <t>Enviado</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -1635,7 +1640,7 @@
         </is>
       </c>
     </row>
-    <row r="22">
+    <row r="22" ht="224" customHeight="1" s="11">
       <c r="A22" t="inlineStr">
         <is>
           <t>2026-08-10</t>
@@ -1666,7 +1671,7 @@
           <t>Afinación profesional de motor diésel (limpieza inyección, turbo, EGR)</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
+      <c r="G22" s="12" t="inlineStr">
         <is>
           <t>Hola! Estamos construyendo Neggo y queremos que un taller como AutoReel haga parte.
 Vi que se especializan en afinación de motor diésel — limpieza de inyección, turbo, EGR, ese nivel de detalle no lo hace cualquier taller en Medellín.
@@ -1676,7 +1681,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Armado</t>
+          <t>Enviado</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -1690,7 +1695,7 @@
         </is>
       </c>
     </row>
-    <row r="23">
+    <row r="23" ht="208" customHeight="1" s="11">
       <c r="A23" t="inlineStr">
         <is>
           <t>2026-08-10</t>
@@ -1721,7 +1726,7 @@
           <t>Contenido de prevención (disco a punto de rayarse), enfoque en revisión preventiva</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="G23" s="12" t="inlineStr">
         <is>
           <t>Hola! Te escribo porque estamos construyendo Neggo y queremos que un taller como Vehifrenos haga parte.
 Vi el video donde muestran el disco a punto de rayarse antes de que sea tarde — ese enfoque en prevención es justo lo que mucha gente no encuentra en un taller.
@@ -1731,7 +1736,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Armado</t>
+          <t>Enviado</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -1745,7 +1750,7 @@
         </is>
       </c>
     </row>
-    <row r="24">
+    <row r="24" ht="224" customHeight="1" s="11">
       <c r="A24" t="inlineStr">
         <is>
           <t>2026-08-10</t>
@@ -1776,7 +1781,7 @@
           <t>50 años de experiencia, alineación/balanceo, frenos, batería, llantas Goodyear/Michelin/BFGoodrich</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
+      <c r="G24" s="12" t="inlineStr">
         <is>
           <t>Buenas tardes. Los 50 años de Autollantas Nutibara ya son una carta de presentación que pocos talleres en Medellín pueden mostrar — no es algo que se pueda inventar.
 Le escribo porque estamos construyendo Neggo, pensado como un complemento a lo que un taller con su trayectoria ya construyó: hoy mucha gente evita probar un taller nuevo por miedo a una mala experiencia (entrar con un problema y salir con tres, sin garantía real). Nosotros verificamos cada taller antes de aparecer en la plataforma, así el cliente llega a ustedes ya con la confianza puesta, no comparando a ciegas contra talleres sin trayectoria.
@@ -1785,7 +1790,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Armado</t>
+          <t>Enviado</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -1799,7 +1804,7 @@
         </is>
       </c>
     </row>
-    <row r="25">
+    <row r="25" ht="208" customHeight="1" s="11">
       <c r="A25" t="inlineStr">
         <is>
           <t>2026-08-10</t>
@@ -1830,7 +1835,7 @@
           <t>Especialistas Audi/Volkswagen, técnicos certificados en marcas premium, 20% dcto primer mantenimiento</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
+      <c r="G25" s="12" t="inlineStr">
         <is>
           <t>Hola! Estamos construyendo Neggo y queremos que un taller como ServiVag haga parte.
 Vi que se especializan en Audi y Volkswagen con técnicos certificados en marcas premium — ese nivel de especialización es exactamente lo que un dueño de un carro de alta gama busca y no siempre encuentra.
@@ -1840,7 +1845,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Armado</t>
+          <t>Enviado</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -1854,7 +1859,7 @@
         </is>
       </c>
     </row>
-    <row r="26">
+    <row r="26" ht="208" customHeight="1" s="11">
       <c r="A26" t="inlineStr">
         <is>
           <t>2026-08-10</t>
@@ -1885,7 +1890,7 @@
           <t>Cambio de aceite desde $98.000, mantenimiento preventivo, lubricación y filtración</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
+      <c r="G26" s="12" t="inlineStr">
         <is>
           <t>Hola! Te escribo porque estamos construyendo Neggo y queremos que un taller como el suyo haga parte.
 Vi que tienen cambio de aceite desde $98.000 con un enfoque real en mantenimiento preventivo — ese tipo de claridad en precio es algo que a muchos clientes les da tranquilidad desde el primer contacto.
@@ -1895,7 +1900,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Armado</t>
+          <t>Enviado</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -1909,7 +1914,7 @@
         </is>
       </c>
     </row>
-    <row r="27">
+    <row r="27" s="11">
       <c r="A27" t="inlineStr">
         <is>
           <t>2026-08-10</t>
@@ -1959,7 +1964,7 @@
         </is>
       </c>
     </row>
-    <row r="28">
+    <row r="28" ht="240" customHeight="1" s="11">
       <c r="A28" t="inlineStr">
         <is>
           <t>2026-08-10</t>
@@ -1990,7 +1995,7 @@
           <t>Ya se posicionan como 'Centro de Servicios Automotriz de Confianza', cuenta verificada, secciones de Casos de Éxito y Testimonios, especialistas Mazda</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
+      <c r="G28" s="12" t="inlineStr">
         <is>
           <t>Hola! Te escribo porque estamos construyendo Neggo y su taller me llamó la atención apenas vi el perfil.
 Ya hablan de ser 'tu Centro de Servicios Automotriz de Confianza' — literalmente lo dice su bio — y tienen hasta una sección de Casos de Éxito y Testimonios. Eso es exactamente lo que Neggo busca resaltar de los talleres que sí trabajan bien.
@@ -2000,7 +2005,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Armado</t>
+          <t>Enviado</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -2014,7 +2019,7 @@
         </is>
       </c>
     </row>
-    <row r="29">
+    <row r="29" ht="208" customHeight="1" s="11">
       <c r="A29" t="inlineStr">
         <is>
           <t>2026-08-10</t>
@@ -2045,7 +2050,7 @@
           <t>Más de 10 años, ya hace parte de una red 'Talleres Aliados / Importadoras Asociadas', revisión general gratis con cambio de aceite</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
+      <c r="G29" s="12" t="inlineStr">
         <is>
           <t>Buenas! Le escribo porque estamos construyendo Neggo y AUTOLEX me pareció un caso interesante — ya hacen parte de una red de Talleres Aliados con Importadoras Asociadas, y tienen más de 10 años cuidando motores en Envigado.
 Eso demuestra algo que Neggo también busca resolver del otro lado: mucha gente no sabe distinguir un taller confiable de uno que no lo es, y termina evitando probar talleres nuevos por miedo a salir con más daños de los que llegó. Nosotros verificamos cada taller antes de listarlo en la plataforma, para que el cliente llegue ya con la confianza puesta — algo que complementa la red que ya construyeron, no la reemplaza.
@@ -2054,21 +2059,30 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Armado</t>
+          <t>Respondió</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Buenas! Con gusto le cuento un poco más.
+Neggo verifica cada negocio antes de mostrarlo en la plataforma, así el cliente que llega hasta ustedes ya sabe que AUTOLEX es un taller real y confiable — no está adivinando entre opciones que prometen lo mismo. Eso complementa la red de Talleres Aliados con Importadoras Asociadas que ya construyeron, no la reemplaza.
+Concretamente: un cliente en Envigado (o en su zona) busca algo puntual — revisión, mantenimiento, un problema específico — y si es un caso que aplica para ustedes, les llega directo con el contacto ya disponible, sin intermediarios.
+Sobre el pago, lo dejamos abierto y lo conversamos según lo que le funcione mejor a AUTOLEX: puede ser pagando por cada cliente que enviamos, o solo cuando ese cliente efectivamente toma el servicio con ustedes. Nada fijo todavía.
+¿Tendría 10-15 minutos esta semana para una llamada corta y le explico todo con calma?</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Esperar a que Jhey lo revise y envíe</t>
+          <t>Esperar respuesta / agendar llamada si acepta</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>CUENTA GRANDE (red de talleres aliados, +10 años) — tono profesional aplicado.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
+          <t>CUENTA GRANDE (red de talleres aliados, +10 años) — tono profesional aplicado. | RESPONDIÓ (10 ago) — pidió más info, se explicó el mecanismo con tono cuenta grande.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="208" customHeight="1" s="11">
       <c r="A30" t="inlineStr">
         <is>
           <t>2026-08-10</t>
@@ -2099,7 +2113,7 @@
           <t>Latonería/pintura de alto nivel (Land Cruiser Prado 2012 actualizada a 2024, body kit, tapizado)</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr">
+      <c r="G30" s="12" t="inlineStr">
         <is>
           <t>Hola! Estamos construyendo Neggo y queremos que un taller como Shopping CARSS haga parte.
 Vi el trabajo que hicieron en la Land Cruiser Prado 2012 actualizada a 2024 — pintura, body kit, tapizado — ese nivel de detalle no lo tiene cualquier taller.
@@ -2109,7 +2123,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Armado</t>
+          <t>Enviado</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -2123,7 +2137,7 @@
         </is>
       </c>
     </row>
-    <row r="31">
+    <row r="31" ht="192" customHeight="1" s="11">
       <c r="A31" t="inlineStr">
         <is>
           <t>2026-08-10</t>
@@ -2154,7 +2168,7 @@
           <t>Servicio de PDR (extracción de golpes sin pintar), cuenta verificada</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
+      <c r="G31" s="12" t="inlineStr">
         <is>
           <t>Hola! Te escribo porque estamos construyendo Neggo y queremos que un taller como Cars System haga parte.
 Vi el servicio de PDR (extracción de golpes sin pintar) — es un servicio que mucha gente ni sabe que existe, y cuando lo necesita no sabe en quién confiar para hacerlo bien.
@@ -2164,7 +2178,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Armado</t>
+          <t>Enviado</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -2173,7 +2187,7 @@
         </is>
       </c>
     </row>
-    <row r="32">
+    <row r="32" ht="192" customHeight="1" s="11">
       <c r="A32" t="inlineStr">
         <is>
           <t>2026-08-10</t>
@@ -2204,7 +2218,7 @@
           <t>15 años de experiencia en rines y llantas, presencia multi-sede en el Área Metropolitana, web propia</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr">
+      <c r="G32" s="12" t="inlineStr">
         <is>
           <t>Buenas! Le escribo porque estamos construyendo Neggo y Todorines me pareció un caso interesante — 15 años de experiencia y presencia en Medellín, Bello, Sabaneta, Envigado e Itagüí no es algo que cualquiera pueda mostrar.
 Le cuento por qué le escribo: mucha gente evita comprar rines o llantas en un lugar que no conoce por miedo a que le vendan algo de mala calidad o mal instalado. Eso frena ventas incluso para negocios como el suyo, con trayectoria real. En Neggo verificamos cada negocio antes de listarlo, así el cliente llega ya con la confianza puesta, sin comparar a ciegas.
@@ -2213,7 +2227,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Armado</t>
+          <t>Enviado</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -2227,7 +2241,7 @@
         </is>
       </c>
     </row>
-    <row r="33">
+    <row r="33" s="11">
       <c r="A33" t="inlineStr">
         <is>
           <t>2026-08-10</t>
@@ -2276,7 +2290,7 @@
         </is>
       </c>
     </row>
-    <row r="34">
+    <row r="34" ht="192" customHeight="1" s="11">
       <c r="A34" t="inlineStr">
         <is>
           <t>2026-08-10</t>
@@ -2307,7 +2321,7 @@
           <t>Domicilio e instalación gratis 24/7, bono de descuento $60.000</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
+      <c r="G34" s="12" t="inlineStr">
         <is>
           <t>Hola! Te escribo porque estamos construyendo Neggo y queremos que un negocio como el suyo haga parte.
 Vi que manejan domicilio e instalación gratis 24/7 en Medellín — para alguien varado con el carro sin batería, esa rapidez es justo lo que necesita, pero también lo que más aprovechan los que no son serios.
@@ -2316,30 +2330,21 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Respondió</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>Hola Daniel! Con gusto te cuento.
-Neggo es una plataforma donde la gente busca negocios de confianza para resolver algo puntual — en tu caso, alguien que necesita cambiar la batería del carro, muchas veces varado o con afán. Nosotros verificamos cada negocio antes de que aparezca en la plataforma, así el cliente que te contacta ya llega confiando en que sos real y serio, no adivinando entre opciones.
-Lo que buscamos con vos es que Baterías a Domicilio 24 Horas esté ahí como una opción verificada — con tu servicio de domicilio e instalación gratis 24/7, que ya es un diferencial fuerte frente a otros.
-El modelo de pago es flexible, lo vemos según lo que te sirva más a vos: podés pagar por cada cliente que te enviamos, o solo cuando ese cliente efectivamente te compra. Nada fijo todavía, lo conversamos según cómo trabajás.
-¿Tenés 10-15 minutos esta semana, una llamada rápida o seguimos por acá, para contarte los detalles completos?</t>
+          <t>Enviado</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Esperar respuesta de Daniel / agendar llamada si acepta</t>
+          <t>Esperar a que Jhey lo revise y envíe</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>Competidor directo de Baterías para carro Medellín — mensaje con gancho distinto (velocidad/domicilio vs. diagnóstico honesto). | RESPONDIÓ (10 ago) — Daniel Marín pidió más info, se le explicó el mecanismo y modelo de pago abierto.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
+          <t>Competidor directo de Baterías para carro Medellín — mensaje con gancho distinto (velocidad/domicilio vs. diagnóstico honesto).</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="160" customHeight="1" s="11">
       <c r="A35" t="inlineStr">
         <is>
           <t>2026-08-10</t>
@@ -2370,7 +2375,7 @@
           <t>Electrónica automotriz</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
+      <c r="G35" s="12" t="inlineStr">
         <is>
           <t>Hola! Estamos construyendo Neggo y queremos que un negocio como Autosafecol haga parte.
 La electrónica de un carro es de lo que más desconfianza genera — mucha gente no sabe si el problema real era lo que le dijeron, o si terminó pagando por algo que no necesitaba.
@@ -2379,7 +2384,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Armado</t>
+          <t>Enviado</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -2408,16 +2413,16 @@
   <dimension ref="A1:K46"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="45" customWidth="1" min="5" max="5"/>
-    <col width="65" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="45" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" style="11" min="1" max="1"/>
+    <col width="22" customWidth="1" style="11" min="2" max="3"/>
+    <col width="40" customWidth="1" style="11" min="4" max="4"/>
+    <col width="45" customWidth="1" style="11" min="5" max="5"/>
+    <col width="65" customWidth="1" style="11" min="6" max="6"/>
+    <col width="16" customWidth="1" style="11" min="7" max="7"/>
+    <col width="45" customWidth="1" style="11" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="56" customHeight="1">
+    <row r="1" ht="56" customHeight="1" s="11">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Fecha</t>
@@ -2474,7 +2479,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="126" customHeight="1">
+    <row r="2" ht="126" customHeight="1" s="11">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
@@ -2526,7 +2531,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="112" customHeight="1">
+    <row r="3" ht="112" customHeight="1" s="11">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
@@ -2578,7 +2583,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="280" customHeight="1">
+    <row r="4" ht="280" customHeight="1" s="11">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
@@ -2630,7 +2635,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="252" customHeight="1">
+    <row r="5" ht="252" customHeight="1" s="11">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
@@ -2682,7 +2687,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="182" customHeight="1">
+    <row r="6" ht="182" customHeight="1" s="11">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
@@ -2734,7 +2739,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="319" customHeight="1">
+    <row r="7" ht="319" customHeight="1" s="11">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
@@ -2786,7 +2791,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="266" customHeight="1">
+    <row r="8" ht="266" customHeight="1" s="11">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
@@ -2838,7 +2843,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="196" customHeight="1">
+    <row r="9" ht="196" customHeight="1" s="11">
       <c r="A9" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
@@ -2890,7 +2895,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="196" customHeight="1">
+    <row r="10" ht="196" customHeight="1" s="11">
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
@@ -2942,7 +2947,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="196" customHeight="1">
+    <row r="11" ht="196" customHeight="1" s="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
@@ -2994,7 +2999,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="196" customHeight="1">
+    <row r="12" ht="196" customHeight="1" s="11">
       <c r="A12" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
@@ -3046,7 +3051,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="196" customHeight="1">
+    <row r="13" ht="196" customHeight="1" s="11">
       <c r="A13" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
@@ -3098,7 +3103,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="154" customHeight="1">
+    <row r="14" ht="154" customHeight="1" s="11">
       <c r="A14" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
@@ -3155,7 +3160,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="293" customHeight="1">
+    <row r="15" ht="293" customHeight="1" s="11">
       <c r="A15" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
@@ -3208,7 +3213,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="168" customHeight="1">
+    <row r="16" ht="168" customHeight="1" s="11">
       <c r="A16" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
@@ -3261,7 +3266,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="384" customHeight="1">
+    <row r="17" ht="384" customHeight="1" s="11">
       <c r="A17" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
@@ -3318,7 +3323,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="352" customHeight="1">
+    <row r="18" ht="352" customHeight="1" s="11">
       <c r="A18" s="2" t="inlineStr">
         <is>
           <t>2026-08-04</t>
@@ -3371,7 +3376,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="358" customHeight="1">
+    <row r="19" ht="358" customHeight="1" s="11">
       <c r="A19" s="2" t="inlineStr">
         <is>
           <t>2026-08-04</t>
@@ -3424,7 +3429,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="376" customHeight="1">
+    <row r="20" ht="376" customHeight="1" s="11">
       <c r="A20" s="2" t="inlineStr">
         <is>
           <t>2026-08-04</t>
@@ -3477,7 +3482,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="324" customHeight="1">
+    <row r="21" ht="324" customHeight="1" s="11">
       <c r="A21" s="2" t="inlineStr">
         <is>
           <t>2026-08-04</t>
@@ -3534,7 +3539,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="714" customHeight="1">
+    <row r="22" ht="409.6" customHeight="1" s="11">
       <c r="A22" s="2" t="inlineStr">
         <is>
           <t>2026-08-04</t>
@@ -3591,7 +3596,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="126" customHeight="1">
+    <row r="23" ht="126" customHeight="1" s="11">
       <c r="A23" s="2" t="inlineStr">
         <is>
           <t>2026-08-04</t>
@@ -3646,7 +3651,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="126" customHeight="1">
+    <row r="24" ht="126" customHeight="1" s="11">
       <c r="A24" s="2" t="inlineStr">
         <is>
           <t>2026-08-04</t>
@@ -3700,7 +3705,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="126" customHeight="1">
+    <row r="25" ht="126" customHeight="1" s="11">
       <c r="A25" s="2" t="inlineStr">
         <is>
           <t>2026-08-04</t>
@@ -3753,7 +3758,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="400" customHeight="1">
+    <row r="26" ht="400" customHeight="1" s="11">
       <c r="A26" s="2" t="inlineStr">
         <is>
           <t>2026-08-05</t>
@@ -3813,7 +3818,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="331.2" customHeight="1">
+    <row r="27" ht="331.25" customHeight="1" s="11">
       <c r="A27" s="2" t="inlineStr">
         <is>
           <t>2026-08-05</t>
@@ -3872,7 +3877,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="278.1" customHeight="1">
+    <row r="28" ht="278" customHeight="1" s="11">
       <c r="A28" s="2" t="inlineStr">
         <is>
           <t>2026-08-05</t>
@@ -3931,7 +3936,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="126" customHeight="1">
+    <row r="29" ht="126" customHeight="1" s="11">
       <c r="A29" s="2" t="inlineStr">
         <is>
           <t>2026-08-06</t>
@@ -3991,7 +3996,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="126" customHeight="1">
+    <row r="30" ht="126" customHeight="1" s="11">
       <c r="A30" s="2" t="inlineStr">
         <is>
           <t>2026-08-06</t>
@@ -4050,7 +4055,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="126" customHeight="1">
+    <row r="31" ht="126" customHeight="1" s="11">
       <c r="A31" s="2" t="inlineStr">
         <is>
           <t>2026-08-06</t>
@@ -4109,7 +4114,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="126" customHeight="1">
+    <row r="32" ht="126" customHeight="1" s="11">
       <c r="A32" s="2" t="inlineStr">
         <is>
           <t>2026-08-06</t>
@@ -4161,7 +4166,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="126" customHeight="1">
+    <row r="33" ht="126" customHeight="1" s="11">
       <c r="A33" s="2" t="inlineStr">
         <is>
           <t>2026-08-06</t>
@@ -4218,7 +4223,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="126" customHeight="1">
+    <row r="34" ht="126" customHeight="1" s="11">
       <c r="A34" s="2" t="inlineStr">
         <is>
           <t>2026-08-06</t>
@@ -4275,7 +4280,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="126" customHeight="1">
+    <row r="35" ht="126" customHeight="1" s="11">
       <c r="A35" s="2" t="inlineStr">
         <is>
           <t>2026-08-07</t>
@@ -4327,7 +4332,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="126" customHeight="1">
+    <row r="36" ht="126" customHeight="1" s="11">
       <c r="A36" s="2" t="inlineStr">
         <is>
           <t>2026-08-07</t>
@@ -4379,7 +4384,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="126" customHeight="1">
+    <row r="37" ht="126" customHeight="1" s="11">
       <c r="A37" s="2" t="inlineStr">
         <is>
           <t>2026-08-07</t>
@@ -4436,7 +4441,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="126" customHeight="1">
+    <row r="38" ht="126" customHeight="1" s="11">
       <c r="A38" s="2" t="inlineStr">
         <is>
           <t>2026-08-07</t>
@@ -4493,7 +4498,7 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="126" customHeight="1">
+    <row r="39" ht="126" customHeight="1" s="11">
       <c r="A39" s="2" t="inlineStr">
         <is>
           <t>2026-08-07</t>
@@ -4550,7 +4555,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="126" customHeight="1">
+    <row r="40" ht="126" customHeight="1" s="11">
       <c r="A40" s="2" t="inlineStr">
         <is>
           <t>2026-08-07</t>
@@ -4607,7 +4612,7 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="126" customHeight="1">
+    <row r="41" ht="126" customHeight="1" s="11">
       <c r="A41" s="2" t="inlineStr">
         <is>
           <t>2026-08-07</t>
@@ -4664,7 +4669,7 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="126" customHeight="1">
+    <row r="42" ht="126" customHeight="1" s="11">
       <c r="A42" s="2" t="inlineStr">
         <is>
           <t>2026-08-07</t>
@@ -4721,7 +4726,7 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="126" customHeight="1">
+    <row r="43" ht="126" customHeight="1" s="11">
       <c r="A43" s="2" t="inlineStr">
         <is>
           <t>2026-08-10</t>
@@ -4778,7 +4783,7 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="126" customHeight="1">
+    <row r="44" ht="126" customHeight="1" s="11">
       <c r="A44" s="2" t="inlineStr">
         <is>
           <t>2026-08-10</t>
@@ -4835,7 +4840,7 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="126" customHeight="1">
+    <row r="45" ht="126" customHeight="1" s="11">
       <c r="A45" s="2" t="inlineStr">
         <is>
           <t>2026-08-10</t>
@@ -4892,7 +4897,7 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="126" customHeight="1">
+    <row r="46" ht="126" customHeight="1" s="11">
       <c r="A46" s="2" t="inlineStr">
         <is>
           <t>2026-08-10</t>
@@ -4964,16 +4969,16 @@
   <dimension ref="A1:J31"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="10.1640625" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="53.1640625" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="19.83203125" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="31.83203125" bestFit="1" customWidth="1" min="5" max="5"/>
-    <col width="39.83203125" bestFit="1" customWidth="1" min="6" max="6"/>
-    <col width="60" customWidth="1" min="7" max="7"/>
-    <col width="22.33203125" bestFit="1" customWidth="1" min="8" max="8"/>
-    <col width="30" bestFit="1" customWidth="1" min="9" max="9"/>
-    <col width="29.83203125" bestFit="1" customWidth="1" min="10" max="10"/>
+    <col width="10.1640625" bestFit="1" customWidth="1" style="11" min="1" max="1"/>
+    <col width="53.1640625" bestFit="1" customWidth="1" style="11" min="2" max="2"/>
+    <col width="19.83203125" bestFit="1" customWidth="1" style="11" min="3" max="3"/>
+    <col width="28" customWidth="1" style="11" min="4" max="4"/>
+    <col width="31.83203125" bestFit="1" customWidth="1" style="11" min="5" max="5"/>
+    <col width="39.83203125" bestFit="1" customWidth="1" style="11" min="6" max="6"/>
+    <col width="60" customWidth="1" style="11" min="7" max="7"/>
+    <col width="22.33203125" bestFit="1" customWidth="1" style="11" min="8" max="8"/>
+    <col width="30" bestFit="1" customWidth="1" style="11" min="9" max="9"/>
+    <col width="29.83203125" bestFit="1" customWidth="1" style="11" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5028,7 +5033,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="126" customHeight="1">
+    <row r="2" ht="126" customHeight="1" s="11">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
@@ -5080,7 +5085,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="126" customHeight="1">
+    <row r="3" ht="126" customHeight="1" s="11">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
@@ -5132,7 +5137,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="154" customHeight="1">
+    <row r="4" ht="154" customHeight="1" s="11">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
@@ -5184,7 +5189,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="126" customHeight="1">
+    <row r="5" ht="126" customHeight="1" s="11">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>2026-08-03</t>
@@ -5236,7 +5241,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="126" customHeight="1">
+    <row r="6" ht="126" customHeight="1" s="11">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>2026-08-04</t>
@@ -5288,7 +5293,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="126" customHeight="1">
+    <row r="7" ht="126" customHeight="1" s="11">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>2026-08-04</t>
@@ -5340,7 +5345,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="126" customHeight="1">
+    <row r="8" ht="126" customHeight="1" s="11">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>2026-08-04</t>
@@ -5392,7 +5397,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="126" customHeight="1">
+    <row r="9" ht="126" customHeight="1" s="11">
       <c r="A9" s="2" t="inlineStr">
         <is>
           <t>2026-08-04</t>
@@ -5444,7 +5449,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="126" customHeight="1">
+    <row r="10" ht="126" customHeight="1" s="11">
       <c r="A10" s="10" t="inlineStr">
         <is>
           <t>2026-08-04</t>
@@ -5496,7 +5501,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="126" customHeight="1">
+    <row r="11" ht="126" customHeight="1" s="11">
       <c r="A11" s="10" t="inlineStr">
         <is>
           <t>2026-08-04</t>
@@ -5548,7 +5553,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="126" customHeight="1">
+    <row r="12" ht="126" customHeight="1" s="11">
       <c r="A12" s="10" t="inlineStr">
         <is>
           <t>2026-08-04</t>
@@ -5600,7 +5605,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="126" customHeight="1">
+    <row r="13" ht="126" customHeight="1" s="11">
       <c r="A13" s="2" t="inlineStr">
         <is>
           <t>2026-08-05</t>
@@ -5652,7 +5657,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="126" customHeight="1">
+    <row r="14" ht="126" customHeight="1" s="11">
       <c r="A14" s="2" t="inlineStr">
         <is>
           <t>2026-08-05</t>
@@ -5704,7 +5709,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="126" customHeight="1">
+    <row r="15" ht="126" customHeight="1" s="11">
       <c r="A15" s="2" t="inlineStr">
         <is>
           <t>2026-08-05</t>
@@ -5756,7 +5761,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="126" customHeight="1">
+    <row r="16" ht="126" customHeight="1" s="11">
       <c r="A16" s="2" t="inlineStr">
         <is>
           <t>2026-08-05</t>
@@ -5808,7 +5813,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="126" customHeight="1">
+    <row r="17" ht="126" customHeight="1" s="11">
       <c r="A17" s="10" t="inlineStr">
         <is>
           <t>2026-08-06</t>
@@ -5860,7 +5865,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="126" customHeight="1">
+    <row r="18" ht="126" customHeight="1" s="11">
       <c r="A18" s="10" t="inlineStr">
         <is>
           <t>2026-08-06</t>
@@ -5912,7 +5917,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="126" customHeight="1">
+    <row r="19" ht="126" customHeight="1" s="11">
       <c r="A19" s="10" t="inlineStr">
         <is>
           <t>2026-08-06</t>
@@ -5964,7 +5969,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="140" customHeight="1">
+    <row r="20" ht="140" customHeight="1" s="11">
       <c r="A20" s="10" t="inlineStr">
         <is>
           <t>2026-08-07</t>
@@ -6016,7 +6021,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="140" customHeight="1">
+    <row r="21" ht="140" customHeight="1" s="11">
       <c r="A21" s="10" t="inlineStr">
         <is>
           <t>2026-08-07</t>
@@ -6068,7 +6073,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="140" customHeight="1">
+    <row r="22" ht="140" customHeight="1" s="11">
       <c r="A22" s="10" t="inlineStr">
         <is>
           <t>2026-08-07</t>
@@ -6120,7 +6125,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="140" customHeight="1">
+    <row r="23" ht="140" customHeight="1" s="11">
       <c r="A23" s="10" t="inlineStr">
         <is>
           <t>2026-08-07</t>
@@ -6172,7 +6177,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="126" customHeight="1">
+    <row r="24" ht="126" customHeight="1" s="11">
       <c r="A24" s="2" t="inlineStr">
         <is>
           <t>2026-08-07</t>
@@ -6224,7 +6229,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="126" customHeight="1">
+    <row r="25" ht="126" customHeight="1" s="11">
       <c r="A25" s="2" t="inlineStr">
         <is>
           <t>2026-08-07</t>
@@ -6276,7 +6281,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="126" customHeight="1">
+    <row r="26" ht="126" customHeight="1" s="11">
       <c r="A26" s="2" t="inlineStr">
         <is>
           <t>2026-08-07</t>
@@ -6328,7 +6333,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="126" customHeight="1">
+    <row r="27" ht="126" customHeight="1" s="11">
       <c r="A27" s="2" t="inlineStr">
         <is>
           <t>2026-08-07</t>
@@ -6380,7 +6385,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="126" customHeight="1">
+    <row r="28" ht="126" customHeight="1" s="11">
       <c r="A28" s="10" t="inlineStr">
         <is>
           <t>2026-08-10</t>
@@ -6432,7 +6437,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="126" customHeight="1">
+    <row r="29" ht="126" customHeight="1" s="11">
       <c r="A29" s="10" t="inlineStr">
         <is>
           <t>2026-08-10</t>
@@ -6484,7 +6489,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="126" customHeight="1">
+    <row r="30" ht="126" customHeight="1" s="11">
       <c r="A30" s="10" t="inlineStr">
         <is>
           <t>2026-08-10</t>
@@ -6536,7 +6541,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="126" customHeight="1">
+    <row r="31" ht="126" customHeight="1" s="11">
       <c r="A31" s="10" t="inlineStr">
         <is>
           <t>2026-08-10</t>

</xml_diff>

<commit_message>
tracker: Autolex (valor concreto) y Cars System (primer contacto) - respuestas armadas
</commit_message>
<xml_diff>
--- a/docs/tracker-prospectos-neggo.xlsx
+++ b/docs/tracker-prospectos-neggo.xlsx
@@ -2064,21 +2064,22 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Buenas! Con gusto le cuento un poco más.
-Neggo verifica cada negocio antes de mostrarlo en la plataforma, así el cliente que llega hasta ustedes ya sabe que AUTOLEX es un taller real y confiable — no está adivinando entre opciones que prometen lo mismo. Eso complementa la red de Talleres Aliados con Importadoras Asociadas que ya construyeron, no la reemplaza.
-Concretamente: un cliente en Envigado (o en su zona) busca algo puntual — revisión, mantenimiento, un problema específico — y si es un caso que aplica para ustedes, les llega directo con el contacto ya disponible, sin intermediarios.
-Sobre el pago, lo dejamos abierto y lo conversamos según lo que le funcione mejor a AUTOLEX: puede ser pagando por cada cliente que enviamos, o solo cuando ese cliente efectivamente toma el servicio con ustedes. Nada fijo todavía.
-¿Tendría 10-15 minutos esta semana para una llamada corta y le explico todo con calma?</t>
+          <t>Claro! Le cuento rápido para que lo vea cuando pueda salir de conducir:
+Por ahora, como parte del lanzamiento, tenemos 3 formas de pago y usted elige la que más le sirva:
+1) Solo Pauta: $10.000 por cada cliente que le enviamos, sin comisión — el cierre de la venta lo hace usted.
+2) Balanceado: $5.000 por cliente + 3% de comisión, pero la comisión solo aplica si ese cliente efectivamente le compra.
+3) Solo Resultados: no paga nada por adelantado, solo el 8% si el cliente termina comprándole a través de Neggo.
+¿Cuál le cuadra mejor para arrancar?</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Esperar respuesta / agendar llamada si acepta</t>
+          <t>Esperar cuál plan elige / confirmar y agendar cierre</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>CUENTA GRANDE (red de talleres aliados, +10 años) — tono profesional aplicado. | RESPONDIÓ (10 ago) — pidió más info, se explicó el mecanismo con tono cuenta grande.</t>
+          <t>CUENTA GRANDE (red de talleres aliados, +10 años) — tono profesional aplicado. | RESPONDIÓ (10 ago) — pidió más info, se explicó el mecanismo con tono cuenta grande. | 10 ago: pidió valor concreto ('nada fijo' ya no alcanzaba). Se ofrecieron 3 valores PILOTO (10k/0%, 5k/3%, 0/8%) — lógicamente consistentes (CPL baja, comisión sube) pero NO vienen de planes_comercio en BD (esos están flageados como inconsistentes en marketing-neggo.md 5.1). Confirmar con Jhey antes de fijarlos como estándar para todos los comercios.</t>
         </is>
       </c>
     </row>
@@ -2178,12 +2179,25 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Enviado</t>
+          <t>Respondió</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Buenas tardes! Le cuento rápido de qué se trata.
+Hoy mucha gente pospone una reparación de golpes (PDR) porque no sabe en qué taller confiar — le da miedo que le dañen más el carro o le cobren de más sin explicarle bien qué le están haciendo.
+Somos Neggo: verificamos cada taller antes de mostrarlo en la plataforma, así el cliente llega hasta ustedes ya confiando en que es un taller real y serio — no adivinando entre opciones.
+Es una forma de traerle clientes nuevos sin que usted tenga que salir a buscarlos. ¿Le cuento cómo funciona el pago? Es bien sencillo.</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Esperar a que Jhey lo revise y envíe</t>
+          <t>Esperar respuesta / tener listos los 3 valores piloto si pregunta por precio</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>10 ago: primer contacto, preguntó 'de qué se trata' — respuesta corta enfocada en el dolor (PDR + desconfianza).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
pricing: fijar valores piloto confirmados por Jhey (planes 12k/6k/0 + Sello 20k flat) y propagar a agente de Ventas
</commit_message>
<xml_diff>
--- a/docs/tracker-prospectos-neggo.xlsx
+++ b/docs/tracker-prospectos-neggo.xlsx
@@ -2066,10 +2066,11 @@
         <is>
           <t>Claro! Le cuento rápido para que lo vea cuando pueda salir de conducir:
 Por ahora, como parte del lanzamiento, tenemos 3 formas de pago y usted elige la que más le sirva:
-1) Solo Pauta: $10.000 por cada cliente que le enviamos, sin comisión — el cierre de la venta lo hace usted.
-2) Balanceado: $5.000 por cliente + 3% de comisión, pero la comisión solo aplica si ese cliente efectivamente le compra.
-3) Solo Resultados: no paga nada por adelantado, solo el 8% si el cliente termina comprándole a través de Neggo.
-¿Cuál le cuadra mejor para arrancar?</t>
+1) Solo Pauta: $12.000 por cada cliente que le enviamos, sin comisión — el cierre de la venta lo hace usted.
+2) Balanceado: $6.000 por cliente + 2,25% de comisión, pero la comisión solo aplica si ese cliente efectivamente le compra.
+3) Solo Resultados: no paga nada por adelantado, solo el 4,1% si el cliente termina comprándole a través de Neggo.
+Además, si quiere, tenemos el Sello de Confianza: una insignia de verificación que le da al cliente la seguridad de que AUTOLEX es un taller real y confiable antes de contactarlo. Cuesta $20.000 al mes.
+¿Cuál de los 3 planes le cuadra mejor para arrancar?</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -2079,7 +2080,7 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>CUENTA GRANDE (red de talleres aliados, +10 años) — tono profesional aplicado. | RESPONDIÓ (10 ago) — pidió más info, se explicó el mecanismo con tono cuenta grande. | 10 ago: pidió valor concreto ('nada fijo' ya no alcanzaba). Se ofrecieron 3 valores PILOTO (10k/0%, 5k/3%, 0/8%) — lógicamente consistentes (CPL baja, comisión sube) pero NO vienen de planes_comercio en BD (esos están flageados como inconsistentes en marketing-neggo.md 5.1). Confirmar con Jhey antes de fijarlos como estándar para todos los comercios.</t>
+          <t>CUENTA GRANDE (red de talleres aliados, +10 años) — tono profesional aplicado. | RESPONDIÓ (10 ago) — pidió más info, se explicó el mecanismo con tono cuenta grande. | 10 ago: pidió valor concreto ('nada fijo' ya no alcanzaba). 10 ago: Jhey confirmó valores oficiales piloto (12k/0%, 6k/2.25%, 0/4.1% + Sello $20.000/mes flat) para usar en TODA prospección — ver marketing-neggo.md 5.1 actualizado.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
pricing/beneficios: Sello obligatorio (no opcional) + Puntos Neggo y Neggo Ads como próximamente, propagado a Ventas
</commit_message>
<xml_diff>
--- a/docs/tracker-prospectos-neggo.xlsx
+++ b/docs/tracker-prospectos-neggo.xlsx
@@ -2069,7 +2069,8 @@
 1) Solo Pauta: $12.000 por cada cliente que le enviamos, sin comisión — el cierre de la venta lo hace usted.
 2) Balanceado: $6.000 por cliente + 2,25% de comisión, pero la comisión solo aplica si ese cliente efectivamente le compra.
 3) Solo Resultados: no paga nada por adelantado, solo el 4,1% si el cliente termina comprándole a través de Neggo.
-Además, si quiere, tenemos el Sello de Confianza: una insignia de verificación que le da al cliente la seguridad de que AUTOLEX es un taller real y confiable antes de contactarlo. Cuesta $20.000 al mes.
+Al afiliarse, el taller queda con el Sello de Confianza (cuesta $20.000 al mes) — no es un extra opcional, es justamente lo que hace que el cliente identifique a AUTOLEX como un taller verificado y de fiar apenas lo ve, antes de escribirle.
+Y le cuento dos cosas que vienen muy pronto, para que las tenga presentes: vamos a lanzar el Programa de Puntos Neggo, donde sus clientes acumulan puntos por comprarle y usted va a poder activar campañas para incentivarlos (doble puntos, primera compra, etc.). Y más adelante se integra Neggo Ads, para que pueda pautar en redes sociales de forma automática desde el mismo panel de Neggo, sin tener que armar la campaña usted mismo.
 ¿Cuál de los 3 planes le cuadra mejor para arrancar?</t>
         </is>
       </c>
@@ -2080,7 +2081,7 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>CUENTA GRANDE (red de talleres aliados, +10 años) — tono profesional aplicado. | RESPONDIÓ (10 ago) — pidió más info, se explicó el mecanismo con tono cuenta grande. | 10 ago: pidió valor concreto ('nada fijo' ya no alcanzaba). 10 ago: Jhey confirmó valores oficiales piloto (12k/0%, 6k/2.25%, 0/4.1% + Sello $20.000/mes flat) para usar en TODA prospección — ver marketing-neggo.md 5.1 actualizado.</t>
+          <t>CUENTA GRANDE (red de talleres aliados, +10 años) — tono profesional aplicado. | RESPONDIÓ (10 ago) — pidió más info, se explicó el mecanismo con tono cuenta grande. | 10 ago: pidió valor concreto ('nada fijo' ya no alcanzaba). 10 ago: Jhey confirmó valores oficiales piloto (12k/0%, 6k/2.25%, 0/4.1% + Sello $20.000/mes flat) para usar en TODA prospección — ver marketing-neggo.md 5.1 actualizado. | Mensaje ampliado 10 ago con Sello obligatorio + Puntos Neggo y Neggo Ads (ambos 'próximamente', ver marketing-neggo.md 5.1.1).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
tracker: Cars System no interesado por ahora - cerrado con cortesía
</commit_message>
<xml_diff>
--- a/docs/tracker-prospectos-neggo.xlsx
+++ b/docs/tracker-prospectos-neggo.xlsx
@@ -2181,25 +2181,22 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Respondió</t>
+          <t>Perdido</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Buenas tardes! Le cuento rápido de qué se trata.
-Hoy mucha gente pospone una reparación de golpes (PDR) porque no sabe en qué taller confiar — le da miedo que le dañen más el carro o le cobren de más sin explicarle bien qué le están haciendo.
-Somos Neggo: verificamos cada taller antes de mostrarlo en la plataforma, así el cliente llega hasta ustedes ya confiando en que es un taller real y serio — no adivinando entre opciones.
-Es una forma de traerle clientes nuevos sin que usted tenga que salir a buscarlos. ¿Le cuento cómo funciona el pago? Es bien sencillo.</t>
+          <t>¡Gracias a usted por tomarse el tiempo de responder! Sin problema, quedamos por acá. Si más adelante le interesa retomarlo, con gusto le vuelvo a contar. Que tenga un excelente día.</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Esperar respuesta / tener listos los 3 valores piloto si pregunta por precio</t>
+          <t>Reintentar contacto en 2-3 meses (no antes)</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>10 ago: primer contacto, preguntó 'de qué se trata' — respuesta corta enfocada en el dolor (PDR + desconfianza).</t>
+          <t>10 ago: primer contacto, preguntó 'de qué se trata' — respuesta corta enfocada en el dolor (PDR + desconfianza). | 10 ago: dijo 'por el momento no estamos interesados' — cerrado con cortesía, sin presión, puerta abierta a futuro.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
tracker: Alma Prana Spa (cuenta grande) respondió 'Me interesa' - respuesta armada
</commit_message>
<xml_diff>
--- a/docs/tracker-prospectos-neggo.xlsx
+++ b/docs/tracker-prospectos-neggo.xlsx
@@ -5084,7 +5084,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Revisar seguimiento sugerido y decidir si enviar</t>
+          <t>Enviar respuesta armada y agendar llamada (cuenta grande, respondió 'Me interesa')</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -5094,7 +5094,7 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Cuenta grande (713 mil seguidores) — igual encaja en ICP Belleza/Spa Medellín, dirección confirmada en bio. Mensaje listo, pendiente de envío por Jhey (no enviado). | SEGUIMIENTO SUGERIDO (2026-08-06): Hola de nuevo — sé que el ritmo de Alma Prana es alto, así que quería retomar brevemente: seguimos viendo demanda real de spa para parejas en Medellín que hoy no se resuelve por un canal directo de leads calificados. Si tienen 5-10 minutos esta semana, les muestro cómo encajaría con las reservas de último minuto que ya vienen impulsando. | (2026-08-10) Seguimiento del 06 ago sigue sin enviarse — ya son 7 días desde el mensaje original. Urge decisión: enviar el seguimiento sugerido o descartar el prospecto.</t>
+          <t>Cuenta grande (713 mil seguidores) — igual encaja en ICP Belleza/Spa Medellín, dirección confirmada en bio. Mensaje listo, pendiente de envío por Jhey (no enviado). | SEGUIMIENTO SUGERIDO (2026-08-06): Hola de nuevo — sé que el ritmo de Alma Prana es alto, así que quería retomar brevemente: seguimos viendo demanda real de spa para parejas en Medellín que hoy no se resuelve por un canal directo de leads calificados. Si tienen 5-10 minutos esta semana, les muestro cómo encajaría con las reservas de último minuto que ya vienen impulsando. | (2026-08-10) Seguimiento del 06 ago sigue sin enviarse — ya son 7 días desde el mensaje original. Urge decisión: enviar el seguimiento sugerido o descartar el prospecto. | RESPONDIÓ (10 ago) — 'Me interesa', compartió 2 WhatsApp (+573003423075 / +573016827948) y dirección. Respuesta armada con tono cuenta grande (sección 6.1), plan de pago 3 opciones (12k/0%, 6k/2.25%, 0/4.1%), Sello obligatorio $20.000/mes, y Neggo Ads como lista de espera (frase segura de estrategia-adquisicion-clientes-neggo.md 6.1). Pendiente de que Jhey la revise y envíe.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
tracker: Clínica Láser de Piel - propuesta por correo reescrita con pricing actualizado y portafolio adjunto
</commit_message>
<xml_diff>
--- a/docs/tracker-prospectos-neggo.xlsx
+++ b/docs/tracker-prospectos-neggo.xlsx
@@ -1058,17 +1058,30 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>CANAL: correo a info@clinicalaserdepiel.com.co (pidieron "portafolio"). Asunto: Propuesta Neggo — leads verificados para Clínica Láser de Piel. Hola, gracias por la respuesta. Les adjunto el portafolio de Neggo: en él vemos seguido que muchas personas posponen un procedimiento por miedo a caer con un negocio poco confiable — es un freno de conversión real. Nosotros resolvemos justo eso verificando cada negocio antes de listarlo, con Sello de Confianza y código anti-phishing, y solo cobramos por resultado (CPL), sin pauta fija. Adjunto también el detalle de cómo funciona. ¿Tienen 10-15 minutos esta semana para una demo? [Adjuntar docs/marca-assets/portafolio-neggo-b2b.pdf]</t>
+          <t>CANAL: CORREO a info@clinicalaserdepiel.com.co (pidieron portafolio para el 'área encargada'). Asunto: Propuesta Neggo — clientes verificados para Clínica Láser de Piel
+Buen día,
+Gracias por la respuesta. Les escribo de parte de Neggo — adjunto el portafolio para que el área encargada pueda revisarlo con calma.
+Hoy es común que alguien posponga un procedimiento estético porque no sabe en qué clínica confiar: teme caer con un lugar que no cumple lo que promete, o que no tenga el respaldo que un procedimiento así merece. Eso frena decisiones incluso para clínicas serias, porque el cliente no tiene cómo distinguirlas a simple vista.
+En Neggo verificamos cada negocio antes de conectarlo con un cliente. Clínica Láser de Piel aparecería con el Sello de Confianza (incluido al afiliarse, $20.000/mes), que es justamente lo que le permite al cliente identificar que está ante un negocio real y respaldado, antes incluso de escribir.
+El pago es sin permanencia y ustedes eligen cómo prefieren pagar:
+- Solo Pauta: $12.000 por cada cliente que les enviamos, sin comisión.
+- Balanceado: $6.000 por cliente + 2,25% de comisión, solo si ese cliente toma el procedimiento.
+- Solo Resultados: $0 por adelantado, solo el 4,1% si el cliente termina tomando el procedimiento con ustedes.
+Quedamos atentos si el área encargada tiene interés en agendar 10-15 minutos esta semana para resolver cualquier duda.
+Saludos,
+Jhey — Fundador, Neggo
+jf.neggo@gmail.com · 302 433 0410 · neggo.co
+[ADJUNTAR: docs/marca-assets/portafolio-neggo-b2b.pdf]</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>2026-08-04 — responder ya (ver Respuesta sugerida)</t>
+          <t>2026-08-10 — enviar correo con portafolio adjunto</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>Mensaje listo — pendiente de envío por Jhey (no enviado) | RESPONDIÓ (04 ago) — gestiona Ventas/Closer. Respuesta sugerida lista. Pendiente de que Jhey la revise y envíe. | Portafolio B2B real ya disponible (docs/marca-assets/portafolio-neggo-b2b.pdf), agregado a la respuesta 4 ago.</t>
+          <t>Mensaje listo — pendiente de envío por Jhey (no enviado) | RESPONDIÓ (04 ago) — gestiona Ventas/Closer. Respuesta sugerida lista. Pendiente de que Jhey la revise y envíe. | Portafolio B2B real ya disponible (docs/marca-assets/portafolio-neggo-b2b.pdf), agregado a la respuesta 4 ago. | 10 ago: propuesta por correo REESCRITA con pricing actualizado (12k/0%, 6k/2.25%, 0/4.1%, Sello obligatorio $20.000/mes) — la versión del 4 ago estaba desactualizada y sin precios concretos.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
crm: nuevo CRM de ventas consolidado (docs/crm-ventas-neggo.xlsx) + tablero visual, reemplaza el tracker de 3 hojas
</commit_message>
<xml_diff>
--- a/docs/tracker-prospectos-neggo.xlsx
+++ b/docs/tracker-prospectos-neggo.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -81,6 +81,14 @@
       <family val="2"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -114,7 +122,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -145,6 +153,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2436,7 +2450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K46"/>
+  <dimension ref="A1:K51"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" style="11" min="1" max="1"/>
@@ -4977,6 +4991,291 @@
       <c r="K46" s="2" t="inlineStr">
         <is>
           <t>EXPLORATORIO — sin pitch formal ni CTA de registro (regla secciones 9-10). 5.784 seguidores, 500+ contactos — no aplica tratamiento de cuenta grande de la sección 6.1 (esa sección rige el pitch de comercios directos, no el segmento exploratorio de Banco-Constructora, mismo criterio ya usado con otros contactos de este segmento en el tracker).</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="126" customHeight="1" s="11">
+      <c r="A47" s="13" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B47" s="13" t="inlineStr">
+        <is>
+          <t>Comercio directo</t>
+        </is>
+      </c>
+      <c r="C47" s="13" t="inlineStr">
+        <is>
+          <t>Luisa María De Moya Ariza</t>
+        </is>
+      </c>
+      <c r="D47" s="13" t="inlineStr">
+        <is>
+          <t>Contadora Pública | Especialista en gestión fiscal y contabilidad pública; CEO — Vuhotravel (agencia de viajes personalizada), Medellín</t>
+        </is>
+      </c>
+      <c r="E47" s="14" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/luisa-mar%C3%ADa-de-moya-ariza-530555150/</t>
+        </is>
+      </c>
+      <c r="F47" s="14" t="inlineStr">
+        <is>
+          <t>Ninguno visible (perfil de 3er grado, vista limitada)</t>
+        </is>
+      </c>
+      <c r="G47" s="13" t="inlineStr">
+        <is>
+          <t>Combina su formación como contadora pública con ser CEO de Vuhotravel, su agencia de viajes personalizada en Medellín — dato tomado del headline verificado del perfil.</t>
+        </is>
+      </c>
+      <c r="H47" s="13" t="inlineStr">
+        <is>
+          <t>Hola, Luisa María. Vi que además de tu trabajo como contadora sos CEO de Vuhotravel, tu agencia de viajes personalizada. Estoy armando Neggo en Medellín: conectamos negocios con clientes que ya están buscando el servicio, y solo pagás cuando el lead es real (CPL bajo, sin pauta ni permanencia). Verificamos cada comercio antes de listarlo, así que a tus clientes les llega con Sello de Confianza. ¿Te cuento en 5 minutos cómo funciona?</t>
+        </is>
+      </c>
+      <c r="I47" s="14" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="J47" s="13" t="inlineStr">
+        <is>
+          <t>Mensaje armado</t>
+        </is>
+      </c>
+      <c r="K47" s="13" t="inlineStr">
+        <is>
+          <t>Categoría: Viaje (segunda de esta categoría en el canal LinkedIn, tenía 1 prospecto previo — Silviana Cardona). Perfil de 3er grado con vista limitada por LinkedIn (362 contactos, sin sección Acerca de ni actividad visible) — el gancho se apoya solo en el headline verificado del perfil, no se inventó ningún dato adicional. Cuenta verificada pero sin señales de "cuenta grande" (362 contactos) — no aplica tratamiento de la sección 6.1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="126" customHeight="1" s="11">
+      <c r="A48" s="13" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B48" s="13" t="inlineStr">
+        <is>
+          <t>Comercio directo</t>
+        </is>
+      </c>
+      <c r="C48" s="13" t="inlineStr">
+        <is>
+          <t>Valeria Upegui Palacio</t>
+        </is>
+      </c>
+      <c r="D48" s="13" t="inlineStr">
+        <is>
+          <t>Gerente Comercial | Administradora de Negocios | Agente Inmobiliaria | Mercado Inmobiliario Internacional, Medellín</t>
+        </is>
+      </c>
+      <c r="E48" s="14" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/valeria-upegui-palacio-50834a73/</t>
+        </is>
+      </c>
+      <c r="F48" s="14" t="inlineStr">
+        <is>
+          <t>Andrés (contacto en común, apellido no confirmado en la vista del perfil)</t>
+        </is>
+      </c>
+      <c r="G48" s="13" t="inlineStr">
+        <is>
+          <t>Trabaja mercado inmobiliario tanto local (Medellín) como internacional — su perfil lista "MV_Realestatefl" como experiencia, vínculo con el mercado de Florida.</t>
+        </is>
+      </c>
+      <c r="H48" s="13" t="inlineStr">
+        <is>
+          <t>Hola, Valeria. Vi tu perfil — manejás mercado inmobiliario tanto local como internacional, con experiencia en Florida. En Neggo conectamos comercios de Medellín con clientes que ya buscan activamente, pagando por resultado real, sin contrato de permanencia. Cada cliente tiene un código de verificación único por sesión, para que sepa que quien lo contacta es realmente vos y no alguien haciéndose pasar por tu inmobiliaria. ¿Charlamos 10 minutos esta semana?</t>
+        </is>
+      </c>
+      <c r="I48" s="14" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="J48" s="13" t="inlineStr">
+        <is>
+          <t>Mensaje armado</t>
+        </is>
+      </c>
+      <c r="K48" s="13" t="inlineStr">
+        <is>
+          <t>Categoría: Vivienda (segunda de esta categoría en el canal LinkedIn, tenía 1 prospecto previo — Juliana Guzman Valencia). Contacto en común mostrado solo como "Andrés" sin apellido confirmado — verificar identidad exacta antes de enviar. 563 seguidores, 500+ contactos — no aplica tratamiento de cuenta grande de la sección 6.1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="126" customHeight="1" s="11">
+      <c r="A49" s="13" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B49" s="13" t="inlineStr">
+        <is>
+          <t>Conector</t>
+        </is>
+      </c>
+      <c r="C49" s="13" t="inlineStr">
+        <is>
+          <t>Andrea Mejía Uribe</t>
+        </is>
+      </c>
+      <c r="D49" s="13" t="inlineStr">
+        <is>
+          <t>Directora de Proyectos | Estratega de Negocios | Consultora de MIPYMES | Abogada — más de 10 años liderando Cultura Estratégica, Colombia</t>
+        </is>
+      </c>
+      <c r="E49" s="14" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/andrea-mej%C3%ADa-uribe-80322596/</t>
+        </is>
+      </c>
+      <c r="F49" s="14" t="inlineStr">
+        <is>
+          <t>Omar (contacto en común, apellido no confirmado en la vista del perfil)</t>
+        </is>
+      </c>
+      <c r="G49" s="13" t="inlineStr">
+        <is>
+          <t>Publicaciones recurrentes en su perfil sobre flujo de caja, registro de marca y asesorías legales/financieras/estratégicas para pymes, acumuladas a lo largo de más de un año de actividad.</t>
+        </is>
+      </c>
+      <c r="H49" s="13" t="inlineStr">
+        <is>
+          <t>Hola, Andrea. Vi tus publicaciones sobre flujo de caja y protección de marca para pymes — se nota la experiencia de más de 10 años asesorando negocios pequeños en temas legales, financieros y comerciales. Estoy construyendo Neggo, una plataforma que conecta comercios de Medellín con clientes verificados y con score financiero real, cobrando solo cuando hay un resultado concreto. Seguro varios de los negocios que has asesorado necesitan más clientes calificados, no solo orden interno — ¿charlamos para ver si tiene sentido referirnos negocios?</t>
+        </is>
+      </c>
+      <c r="I49" s="14" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="J49" s="13" t="inlineStr">
+        <is>
+          <t>Mensaje armado</t>
+        </is>
+      </c>
+      <c r="K49" s="13" t="inlineStr">
+        <is>
+          <t>Canal Conector. En un post de hace ~1 año menciona estar buscando un rol corporativo in-house — el mensaje evita asumir que Cultura Estratégica sigue siendo su actividad principal hoy y se apoya en su trayectoria de +10 años asesorando pymes, no en el estado actual de la empresa. Verificar identidad exacta del contacto en común "Omar" antes de enviar. Perfil verificado, 1.434 seguidores — no aplica tratamiento de cuenta grande de la sección 6.1 (esa sección rige el pitch a comercios directos, no el canal Conector).</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="126" customHeight="1" s="11">
+      <c r="A50" s="13" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B50" s="13" t="inlineStr">
+        <is>
+          <t>Conector</t>
+        </is>
+      </c>
+      <c r="C50" s="13" t="inlineStr">
+        <is>
+          <t>Alejandro Betancur Ríos</t>
+        </is>
+      </c>
+      <c r="D50" s="13" t="inlineStr">
+        <is>
+          <t>Consultor | Mentor | Marketing | Ventas | Formación Comercial — Fundador de 4AZUL "Entrenamiento en Marketing y Ventas"; docente en Institución Universitaria ESUMER, Medellín</t>
+        </is>
+      </c>
+      <c r="E50" s="14" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/alejandro-betancur-rios/</t>
+        </is>
+      </c>
+      <c r="F50" s="14" t="inlineStr">
+        <is>
+          <t>Manuela, Laura (contactos en común, apellidos no confirmados en la vista del perfil)</t>
+        </is>
+      </c>
+      <c r="G50" s="13" t="inlineStr">
+        <is>
+          <t>Dirige 4AZUL, su propia empresa de entrenamiento en marketing y ventas, y es docente en ESUMER — datos tomados del headline y la experiencia listada en su perfil.</t>
+        </is>
+      </c>
+      <c r="H50" s="13" t="inlineStr">
+        <is>
+          <t>Hola, Alejandro. Vi que además de dar clases en ESUMER lideras 4AZUL, formando equipos comerciales en marketing y ventas. Estoy armando Neggo: conectamos comercios de Medellín con clientes que ya están buscando el servicio, con score financiero visible y pago solo por resultado real. Imagino que varios de los negocios que entrenás en ventas están buscando más leads calificados, no solo mejorar el cierre. ¿Tenés 10 minutos para ver si nos conviene referirnos clientes?</t>
+        </is>
+      </c>
+      <c r="I50" s="14" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="J50" s="13" t="inlineStr">
+        <is>
+          <t>Mensaje armado</t>
+        </is>
+      </c>
+      <c r="K50" s="13" t="inlineStr">
+        <is>
+          <t>Canal Conector. Contactos en común mostrados solo con nombre de pila ("Manuela", "Laura"), sin apellido — verificar identidad antes de enviar. 2.810 seguidores, 500+ contactos — no aplica tratamiento de cuenta grande de la sección 6.1 (esa sección rige el pitch a comercios directos, no el canal Conector).</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="126" customHeight="1" s="11">
+      <c r="A51" s="13" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B51" s="13" t="inlineStr">
+        <is>
+          <t>Banco-Constructora</t>
+        </is>
+      </c>
+      <c r="C51" s="13" t="inlineStr">
+        <is>
+          <t>Julián dos Santos</t>
+        </is>
+      </c>
+      <c r="D51" s="13" t="inlineStr">
+        <is>
+          <t>Gerente de Negocios | Engenharia Civil | Ing. Civil (formado en Universidade Paulista, Brasil), Medellín</t>
+        </is>
+      </c>
+      <c r="E51" s="14" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/julian-dos-santos/</t>
+        </is>
+      </c>
+      <c r="F51" s="14" t="inlineStr">
+        <is>
+          <t>Mónica, Omar (contactos en común, apellidos no confirmados en la vista del perfil)</t>
+        </is>
+      </c>
+      <c r="G51" s="13" t="inlineStr">
+        <is>
+          <t>Ingeniero civil formado en Brasil (Universidade Paulista) que hoy trabaja como Gerente de Negocios en el sector construcción en Medellín — dato tomado del headline y la educación listada en su perfil verificado.</t>
+        </is>
+      </c>
+      <c r="H51" s="13" t="inlineStr">
+        <is>
+          <t>Hola, Julián. Vi tu perfil — ingeniero civil formado en Brasil (Universidade Paulista) y ahora Gerente de Negocios acá en Medellín, una combinación poco común. Soy fundador de Neggo, estamos armando un modelo de matching entre comercios, constructoras y bancos en la ciudad — todavía en etapa temprana con constructoras, nada formal por ahora. Me gustaría conocer tu mirada del sector desde tu experiencia, ¿te copás a tomar un café o hablar 15 minutos en algún momento?</t>
+        </is>
+      </c>
+      <c r="I51" s="14" t="inlineStr">
+        <is>
+          <t>Esperar a que Jhey lo envíe</t>
+        </is>
+      </c>
+      <c r="J51" s="13" t="inlineStr">
+        <is>
+          <t>Mensaje armado</t>
+        </is>
+      </c>
+      <c r="K51" s="13" t="inlineStr">
+        <is>
+          <t>EXPLORATORIO — sin pitch formal ni CTA de registro (regla secciones 9-10, Fase 2 Constructoras sigue bloqueada hasta tener 5-10 comercios activos con leads entregados). 2.612 seguidores, cuenta verificada — no aplica tratamiento de cuenta grande de la sección 6.1 (esa sección rige el pitch de comercios directos, no el segmento exploratorio de Banco-Constructora, mismo criterio usado con otros contactos de este segmento en el tracker). Contactos en común mostrados solo con nombre de pila, sin apellido confirmado — verificar antes de enviar.</t>
         </is>
       </c>
     </row>

</xml_diff>